<commit_message>
Tier 1 and Tier 2 filtering active. Ability to pass incomplete data. Obtain close values for TBABH and AB.
</commit_message>
<xml_diff>
--- a/MTGPR_train.xlsx
+++ b/MTGPR_train.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BF0DD66-B3B3-4CF8-9EA8-5A758524FDE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB52E98-A14D-4C1B-833B-67AFECD6D4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1230" yWindow="690" windowWidth="21600" windowHeight="14715" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="91">
   <si>
     <t>tetrabutylammonium bromide</t>
   </si>
@@ -173,9 +173,6 @@
     <t>acetonitrile</t>
   </si>
   <si>
-    <t>Not Found</t>
-  </si>
-  <si>
     <t>ethyl bromide</t>
   </si>
   <si>
@@ -231,6 +228,90 @@
   </si>
   <si>
     <t>tetrapropylammonium iodide</t>
+  </si>
+  <si>
+    <t>CC#N</t>
+  </si>
+  <si>
+    <t>CCC#N</t>
+  </si>
+  <si>
+    <t>[B-](C1=CC=CC=C1)(C2=CC=CC=C2)(C3=CC=CC=C3)C4=CC=CC=C4.CCCC[N+](CCCC)(CCCC)CCCC</t>
+  </si>
+  <si>
+    <t>CC[N+](CC)(CC)CC.[I-]</t>
+  </si>
+  <si>
+    <t>CC[N+](CC)(CC)CC.[N+](=O)([O-])[O-]</t>
+  </si>
+  <si>
+    <t>CCCCCCC[N+](CCCCCCC)(CCCCCCC)CCCCCCC.[Cl-]</t>
+  </si>
+  <si>
+    <t>CCCCCC[N+](CCCCCC)(CCCCCC)CCCCCC.[Br-]</t>
+  </si>
+  <si>
+    <t>C[N+](C)(C)C.[Br-]</t>
+  </si>
+  <si>
+    <t>C[N+](C)(C)C.[I-]</t>
+  </si>
+  <si>
+    <t>CCCCC[N+](CCCCC)(CCCCC)CCCCC.[Br-]</t>
+  </si>
+  <si>
+    <t>CCCCC[N+](CCCCC)(CCCCC)CCCCC.[Cl-]</t>
+  </si>
+  <si>
+    <t>CCCCC[N+](CCCCC)(CCCCC)CCCCC.[I-]</t>
+  </si>
+  <si>
+    <t>CCC[N+](CCC)(CCC)CCC.[Br-]</t>
+  </si>
+  <si>
+    <t>CCC[N+](CCC)(CCC)CCC.[I-]</t>
+  </si>
+  <si>
+    <t>benzonitrile</t>
+  </si>
+  <si>
+    <t>C1=CC=C(C=C1)C#N</t>
+  </si>
+  <si>
+    <t>butanenitrile</t>
+  </si>
+  <si>
+    <t>CCCC#N</t>
+  </si>
+  <si>
+    <t>cyanogen</t>
+  </si>
+  <si>
+    <t>C(#N)C#N</t>
+  </si>
+  <si>
+    <t>dimethylhydrazine</t>
+  </si>
+  <si>
+    <t>CN(C)N</t>
+  </si>
+  <si>
+    <t>dinitrogen tetroxide</t>
+  </si>
+  <si>
+    <t>[N+](=O)([N+](=O)[O-])[O-]</t>
+  </si>
+  <si>
+    <t>hydrazine</t>
+  </si>
+  <si>
+    <t>NN</t>
+  </si>
+  <si>
+    <t>monomethylhydrazine</t>
+  </si>
+  <si>
+    <t>CNN</t>
   </si>
 </sst>
 </file>
@@ -638,7 +719,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -664,7 +745,7 @@
         <v>43</v>
       </c>
       <c r="C2" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="D2">
         <v>228</v>
@@ -731,34 +812,34 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>77</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>78</v>
       </c>
       <c r="D4">
-        <v>179.32</v>
-      </c>
-      <c r="E4">
-        <v>1.3349157276772183</v>
+        <v>263</v>
+      </c>
+      <c r="E4" t="s">
+        <v>2</v>
       </c>
       <c r="F4">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G4">
-        <v>5.9405000000000001</v>
+        <v>10.98</v>
       </c>
       <c r="H4">
-        <v>7.0710678118615568E-4</v>
+        <v>0</v>
       </c>
       <c r="I4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J4" s="2">
-        <v>-21.4</v>
+        <v>163.19999999999999</v>
       </c>
       <c r="K4" s="2">
-        <v>3.3941125496954587</v>
+        <v>0</v>
       </c>
       <c r="L4">
         <v>2</v>
@@ -766,162 +847,162 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>79</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="D5">
-        <v>95.1</v>
+        <v>160.91</v>
       </c>
       <c r="E5">
-        <v>8.3438600180012585</v>
+        <v>0.52844110362461461</v>
       </c>
       <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="G5">
-        <v>2.8133333333333339</v>
-      </c>
-      <c r="H5">
-        <v>3.7846179904097832E-2</v>
+        <v>5</v>
+      </c>
+      <c r="G5" t="s">
+        <v>2</v>
+      </c>
+      <c r="H5" t="s">
+        <v>2</v>
       </c>
       <c r="I5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J5" s="2">
-        <v>-84.15666666666668</v>
-      </c>
-      <c r="K5" s="2">
-        <v>0.45566800780100331</v>
+        <v>-5.8</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L5">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>82</v>
       </c>
       <c r="D6">
-        <v>155</v>
-      </c>
-      <c r="E6" t="s">
-        <v>2</v>
+        <v>245.31</v>
+      </c>
+      <c r="E6">
+        <v>1.4142135623718088E-2</v>
       </c>
       <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6" t="s">
-        <v>2</v>
-      </c>
-      <c r="H6" t="s">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="G6">
+        <v>8.1095000000000006</v>
+      </c>
+      <c r="H6">
+        <v>7.0710678118615568E-4</v>
       </c>
       <c r="I6">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J6" s="2">
-        <v>-95.5</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>2</v>
+        <v>296.91750000000002</v>
+      </c>
+      <c r="K6" s="2">
+        <v>22.637415009963771</v>
       </c>
       <c r="L6">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D7">
-        <v>134.76249999999999</v>
+        <v>179.32</v>
       </c>
       <c r="E7">
-        <v>2.4581073342445094</v>
+        <v>1.3349157276772183</v>
       </c>
       <c r="F7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G7">
-        <v>4.4510000000000005</v>
+        <v>5.9405000000000001</v>
       </c>
       <c r="H7">
-        <v>1.4142135623729393E-3</v>
+        <v>7.0710678118615568E-4</v>
       </c>
       <c r="I7">
         <v>2</v>
       </c>
       <c r="J7" s="2">
-        <v>-137</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>2</v>
+        <v>-21.4</v>
+      </c>
+      <c r="K7" s="2">
+        <v>3.3941125496954587</v>
       </c>
       <c r="L7">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="C8" t="s">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="D8">
-        <v>162.17500000000001</v>
+        <v>215.97499999999999</v>
       </c>
       <c r="E8">
-        <v>0.17677669529663689</v>
+        <v>3.5355339059335411E-2</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
-      <c r="G8" t="s">
-        <v>2</v>
-      </c>
-      <c r="H8" t="s">
-        <v>2</v>
+      <c r="G8">
+        <v>10.071300000000001</v>
+      </c>
+      <c r="H8">
+        <v>1.838477631084507E-3</v>
       </c>
       <c r="I8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J8" s="2">
-        <v>-37.866666666666667</v>
-      </c>
-      <c r="K8" s="2">
-        <v>2.4906491790963527</v>
+        <v>48.3</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L8">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="D9">
-        <v>89.72</v>
-      </c>
-      <c r="E9">
-        <v>2.2642879675518288</v>
+        <v>263.84999999999997</v>
+      </c>
+      <c r="E9" t="s">
+        <v>2</v>
       </c>
       <c r="F9">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G9">
-        <v>0.93920000000000003</v>
+        <v>14.65</v>
       </c>
       <c r="H9" t="s">
         <v>2</v>
@@ -930,77 +1011,77 @@
         <v>1</v>
       </c>
       <c r="J9" s="2">
-        <v>-74.444000000000003</v>
-      </c>
-      <c r="K9" s="2">
-        <v>0.60492148250826439</v>
+        <v>9.08</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L9">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D10">
-        <v>179.5</v>
-      </c>
-      <c r="E10" t="s">
-        <v>2</v>
+        <v>95.1</v>
+      </c>
+      <c r="E10">
+        <v>8.3438600180012585</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10">
-        <v>5.98</v>
-      </c>
-      <c r="H10" t="s">
-        <v>2</v>
+        <v>2.8133333333333339</v>
+      </c>
+      <c r="H10">
+        <v>3.7846179904097832E-2</v>
       </c>
       <c r="I10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J10" s="2">
-        <v>-60.6</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>2</v>
+        <v>-84.15666666666668</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0.45566800780100331</v>
       </c>
       <c r="L10">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="D11">
-        <v>178.01666666666665</v>
-      </c>
-      <c r="E11">
-        <v>3.4822167269331912</v>
+        <v>155</v>
+      </c>
+      <c r="E11" t="s">
+        <v>2</v>
       </c>
       <c r="F11">
-        <v>3</v>
-      </c>
-      <c r="G11">
-        <v>6.4254999999999995</v>
-      </c>
-      <c r="H11">
-        <v>7.778174593052108E-3</v>
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>2</v>
+      </c>
+      <c r="H11" t="s">
+        <v>2</v>
       </c>
       <c r="I11">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J11" s="2">
-        <v>-102.4</v>
+        <v>-95.5</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>2</v>
@@ -1011,101 +1092,101 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D12">
-        <v>207.39999999999998</v>
+        <v>134.76249999999999</v>
       </c>
       <c r="E12">
-        <v>0.98994949366117058</v>
+        <v>2.4581073342445094</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G12">
-        <v>9.1199999999999992</v>
-      </c>
-      <c r="H12" t="s">
-        <v>2</v>
+        <v>4.4510000000000005</v>
+      </c>
+      <c r="H12">
+        <v>1.4142135623729393E-3</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J12" s="2">
-        <v>-12.8</v>
-      </c>
-      <c r="K12" s="2">
-        <v>1.1313708498984758</v>
+        <v>-137</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L12">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>37</v>
+        <v>46</v>
       </c>
       <c r="C13" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D13">
-        <v>179.93333333333331</v>
+        <v>162.17500000000001</v>
       </c>
       <c r="E13">
-        <v>0.20207259421638213</v>
+        <v>0.17677669529663689</v>
       </c>
       <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13" t="s">
+        <v>2</v>
+      </c>
+      <c r="H13" t="s">
+        <v>2</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2">
+        <v>-37.866666666666667</v>
+      </c>
+      <c r="K13" s="2">
+        <v>2.4906491790963527</v>
+      </c>
+      <c r="L13">
         <v>3</v>
-      </c>
-      <c r="G13">
-        <v>6.1319999999999997</v>
-      </c>
-      <c r="H13">
-        <v>2.8284271247465066E-3</v>
-      </c>
-      <c r="I13">
-        <v>2</v>
-      </c>
-      <c r="J13" s="2">
-        <v>-17.850000000000001</v>
-      </c>
-      <c r="K13" s="2">
-        <v>7.9903066274079748</v>
-      </c>
-      <c r="L13">
-        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>49</v>
+        <v>87</v>
       </c>
       <c r="C14" t="s">
-        <v>44</v>
+        <v>88</v>
       </c>
       <c r="D14">
-        <v>180</v>
-      </c>
-      <c r="E14" t="s">
-        <v>2</v>
+        <v>274.93333333333334</v>
+      </c>
+      <c r="E14">
+        <v>0.25658007197234717</v>
       </c>
       <c r="F14">
-        <v>1</v>
-      </c>
-      <c r="G14">
-        <v>5.03</v>
+        <v>3</v>
+      </c>
+      <c r="G14" t="s">
+        <v>2</v>
       </c>
       <c r="H14" t="s">
         <v>2</v>
       </c>
       <c r="I14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J14" s="2">
-        <v>15.5</v>
+        <v>50.63</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>2</v>
@@ -1116,127 +1197,127 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="C15" t="s">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="D15">
-        <v>190.15</v>
-      </c>
-      <c r="E15" t="s">
-        <v>2</v>
+        <v>89.72</v>
+      </c>
+      <c r="E15">
+        <v>2.2642879675518288</v>
       </c>
       <c r="F15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G15">
-        <v>10.856400000000001</v>
-      </c>
-      <c r="H15">
-        <v>0.20040928122220297</v>
+        <v>0.93920000000000003</v>
+      </c>
+      <c r="H15" t="s">
+        <v>2</v>
       </c>
       <c r="I15">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J15" s="2">
-        <v>-119.75</v>
+        <v>-74.444000000000003</v>
       </c>
       <c r="K15" s="2">
-        <v>25.809397513308983</v>
+        <v>0.60492148250826439</v>
       </c>
       <c r="L15">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="C16" t="s">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="D16">
-        <v>395.07499999999999</v>
-      </c>
-      <c r="E16">
-        <v>0.10606601717796604</v>
+        <v>179.5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>2</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G16">
-        <v>15.8154</v>
-      </c>
-      <c r="H16">
-        <v>0.47319585797003511</v>
+        <v>5.98</v>
+      </c>
+      <c r="H16" t="s">
+        <v>2</v>
       </c>
       <c r="I16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J16" s="2">
-        <v>-477.65</v>
-      </c>
-      <c r="K16" s="2">
-        <v>88.600479682674319</v>
+        <v>-60.6</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L16">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="D17">
-        <v>314.14999999999998</v>
-      </c>
-      <c r="E17" t="s">
-        <v>2</v>
+        <v>178.01666666666665</v>
+      </c>
+      <c r="E17">
+        <v>3.4822167269331912</v>
       </c>
       <c r="F17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G17">
-        <v>20.501600000000003</v>
-      </c>
-      <c r="H17" t="s">
-        <v>2</v>
+        <v>6.4254999999999995</v>
+      </c>
+      <c r="H17">
+        <v>7.778174593052108E-3</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J17" s="2">
-        <v>-549.4</v>
-      </c>
-      <c r="K17" s="2">
-        <v>21.778888860545631</v>
+        <v>-102.4</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L17">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>3</v>
+        <v>35</v>
       </c>
       <c r="C18" t="s">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="D18">
-        <v>419.15</v>
-      </c>
-      <c r="E18" t="s">
-        <v>2</v>
+        <v>207.39999999999998</v>
+      </c>
+      <c r="E18">
+        <v>0.98994949366117058</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G18">
-        <v>9.6231999999999989</v>
+        <v>9.1199999999999992</v>
       </c>
       <c r="H18" t="s">
         <v>2</v>
@@ -1245,10 +1326,10 @@
         <v>1</v>
       </c>
       <c r="J18" s="2">
-        <v>-479.3</v>
+        <v>-12.8</v>
       </c>
       <c r="K18" s="2">
-        <v>27.294321753800752</v>
+        <v>1.1313708498984758</v>
       </c>
       <c r="L18">
         <v>2</v>
@@ -1256,83 +1337,83 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="C19" t="s">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="D19">
-        <v>389.9666666666667</v>
+        <v>179.93333333333331</v>
       </c>
       <c r="E19">
-        <v>1.9857828011475314</v>
+        <v>0.20207259421638213</v>
       </c>
       <c r="F19">
         <v>3</v>
       </c>
       <c r="G19">
-        <v>14.95</v>
+        <v>6.1319999999999997</v>
       </c>
       <c r="H19">
-        <v>0.91923881554251108</v>
+        <v>2.8284271247465066E-3</v>
       </c>
       <c r="I19">
         <v>2</v>
       </c>
       <c r="J19" s="2">
-        <v>-600.20000000000005</v>
-      </c>
-      <c r="K19" s="2" t="s">
-        <v>2</v>
+        <v>-17.850000000000001</v>
+      </c>
+      <c r="K19" s="2">
+        <v>7.9903066274079748</v>
       </c>
       <c r="L19">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="C20" t="s">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="D20">
-        <v>502.2</v>
-      </c>
-      <c r="E20" t="s">
-        <v>2</v>
+        <v>220.79500000000002</v>
+      </c>
+      <c r="E20">
+        <v>7.0710678118791415E-3</v>
       </c>
       <c r="F20">
-        <v>1</v>
-      </c>
-      <c r="G20" t="s">
-        <v>2</v>
-      </c>
-      <c r="H20" t="s">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="G20">
+        <v>10.419</v>
+      </c>
+      <c r="H20">
+        <v>1.4142135623735675E-3</v>
       </c>
       <c r="I20">
-        <v>0</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="J20" s="2">
+        <v>54.14</v>
       </c>
       <c r="K20" s="2" t="s">
         <v>2</v>
       </c>
       <c r="L20">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>64</v>
       </c>
       <c r="D21">
-        <v>447</v>
+        <v>180</v>
       </c>
       <c r="E21" t="s">
         <v>2</v>
@@ -1341,7 +1422,7 @@
         <v>1</v>
       </c>
       <c r="G21">
-        <v>20.3</v>
+        <v>5.03</v>
       </c>
       <c r="H21" t="s">
         <v>2</v>
@@ -1350,24 +1431,24 @@
         <v>1</v>
       </c>
       <c r="J21">
-        <v>-363.45</v>
-      </c>
-      <c r="K21">
-        <v>15.700212312789498</v>
+        <v>15.5</v>
+      </c>
+      <c r="K21" t="s">
+        <v>2</v>
       </c>
       <c r="L21">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="C22" t="s">
-        <v>18</v>
+        <v>40</v>
       </c>
       <c r="D22">
-        <v>526.78</v>
+        <v>190.15</v>
       </c>
       <c r="E22" t="s">
         <v>2</v>
@@ -1376,103 +1457,103 @@
         <v>1</v>
       </c>
       <c r="G22">
-        <v>51.24</v>
-      </c>
-      <c r="H22" t="s">
-        <v>2</v>
+        <v>10.856400000000001</v>
+      </c>
+      <c r="H22">
+        <v>0.20040928122220297</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J22">
-        <v>-396.29999999999995</v>
+        <v>-119.75</v>
       </c>
       <c r="K22">
-        <v>18.966988866624746</v>
+        <v>25.809397513308983</v>
       </c>
       <c r="L22">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="C23" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" t="s">
-        <v>2</v>
-      </c>
-      <c r="E23" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D23">
+        <v>395.07499999999999</v>
+      </c>
+      <c r="E23">
+        <v>0.10606601717796604</v>
       </c>
       <c r="F23">
-        <v>0</v>
-      </c>
-      <c r="G23" t="s">
-        <v>2</v>
-      </c>
-      <c r="H23" t="s">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="G23">
+        <v>15.8154</v>
+      </c>
+      <c r="H23">
+        <v>0.47319585797003511</v>
       </c>
       <c r="I23">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J23">
-        <v>-316.17500000000001</v>
+        <v>-477.65</v>
       </c>
       <c r="K23">
-        <v>12.790198069876276</v>
+        <v>88.600479682674319</v>
       </c>
       <c r="L23">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C24" t="s">
-        <v>44</v>
-      </c>
-      <c r="D24" t="s">
-        <v>2</v>
+        <v>50</v>
+      </c>
+      <c r="D24">
+        <v>314.14999999999998</v>
       </c>
       <c r="E24" t="s">
         <v>2</v>
       </c>
       <c r="F24">
-        <v>0</v>
-      </c>
-      <c r="G24" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G24">
+        <v>20.501600000000003</v>
       </c>
       <c r="H24" t="s">
         <v>2</v>
       </c>
       <c r="I24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J24">
-        <v>-430.83333333333331</v>
+        <v>-549.4</v>
       </c>
       <c r="K24">
-        <v>2.2546248764114472</v>
+        <v>21.778888860545631</v>
       </c>
       <c r="L24">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>55</v>
+        <v>3</v>
       </c>
       <c r="C25" t="s">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="D25">
-        <v>264.14999999999998</v>
+        <v>419.15</v>
       </c>
       <c r="E25" t="s">
         <v>2</v>
@@ -1480,75 +1561,75 @@
       <c r="F25">
         <v>1</v>
       </c>
-      <c r="G25" t="s">
-        <v>2</v>
+      <c r="G25">
+        <v>9.6231999999999989</v>
       </c>
       <c r="H25" t="s">
         <v>2</v>
       </c>
       <c r="I25">
-        <v>0</v>
-      </c>
-      <c r="J25" t="s">
-        <v>2</v>
-      </c>
-      <c r="K25" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="J25">
+        <v>-479.3</v>
+      </c>
+      <c r="K25">
+        <v>27.294321753800752</v>
       </c>
       <c r="L25">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>56</v>
+        <v>5</v>
       </c>
       <c r="C26" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="D26">
-        <v>377.15</v>
-      </c>
-      <c r="E26" t="s">
-        <v>2</v>
+        <v>389.9666666666667</v>
+      </c>
+      <c r="E26">
+        <v>1.9857828011475314</v>
       </c>
       <c r="F26">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G26">
-        <v>15.8992</v>
-      </c>
-      <c r="H26" t="s">
-        <v>2</v>
+        <v>14.95</v>
+      </c>
+      <c r="H26">
+        <v>0.91923881554251108</v>
       </c>
       <c r="I26">
-        <v>1</v>
-      </c>
-      <c r="J26" t="s">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="J26">
+        <v>-600.20000000000005</v>
       </c>
       <c r="K26" t="s">
         <v>2</v>
       </c>
       <c r="L26">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C27" t="s">
-        <v>44</v>
-      </c>
-      <c r="D27" t="s">
-        <v>2</v>
+        <v>65</v>
+      </c>
+      <c r="D27">
+        <v>502.2</v>
       </c>
       <c r="E27" t="s">
         <v>2</v>
       </c>
       <c r="F27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" t="s">
         <v>2</v>
@@ -1559,34 +1640,34 @@
       <c r="I27">
         <v>0</v>
       </c>
-      <c r="J27">
-        <v>-256.83333333333331</v>
-      </c>
-      <c r="K27">
-        <v>9.6738479072876338</v>
+      <c r="J27" t="s">
+        <v>2</v>
+      </c>
+      <c r="K27" t="s">
+        <v>2</v>
       </c>
       <c r="L27">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C28" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="D28">
-        <v>653.01</v>
-      </c>
-      <c r="E28">
-        <v>56.766532393656014</v>
+        <v>447</v>
+      </c>
+      <c r="E28" t="s">
+        <v>2</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G28">
-        <v>20.49</v>
+        <v>20.3</v>
       </c>
       <c r="H28" t="s">
         <v>2</v>
@@ -1595,80 +1676,80 @@
         <v>1</v>
       </c>
       <c r="J28">
-        <v>-274.8</v>
+        <v>-363.45</v>
       </c>
       <c r="K28">
-        <v>2.4331050121192805</v>
+        <v>15.700212312789498</v>
       </c>
       <c r="L28">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="C29" t="s">
-        <v>44</v>
-      </c>
-      <c r="D29" t="s">
-        <v>2</v>
+        <v>18</v>
+      </c>
+      <c r="D29">
+        <v>526.78</v>
       </c>
       <c r="E29" t="s">
         <v>2</v>
       </c>
       <c r="F29">
-        <v>0</v>
-      </c>
-      <c r="G29" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G29">
+        <v>51.24</v>
       </c>
       <c r="H29" t="s">
         <v>2</v>
       </c>
       <c r="I29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J29">
-        <v>-199.13333333333333</v>
+        <v>-396.29999999999995</v>
       </c>
       <c r="K29">
-        <v>7.9122268251948746</v>
+        <v>18.966988866624746</v>
       </c>
       <c r="L29">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="C30" t="s">
-        <v>8</v>
-      </c>
-      <c r="D30">
-        <v>683</v>
+        <v>66</v>
+      </c>
+      <c r="D30" t="s">
+        <v>2</v>
       </c>
       <c r="E30" t="s">
         <v>2</v>
       </c>
       <c r="F30">
-        <v>1</v>
-      </c>
-      <c r="G30">
-        <v>37.200000000000003</v>
+        <v>0</v>
+      </c>
+      <c r="G30" t="s">
+        <v>2</v>
       </c>
       <c r="H30" t="s">
         <v>2</v>
       </c>
       <c r="I30">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J30">
-        <v>-330.4</v>
+        <v>-316.17500000000001</v>
       </c>
       <c r="K30">
-        <v>1.4071247279470325</v>
+        <v>12.790198069876276</v>
       </c>
       <c r="L30">
         <v>4</v>
@@ -1676,48 +1757,48 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C31" t="s">
-        <v>44</v>
-      </c>
-      <c r="D31">
-        <v>376.15</v>
+        <v>67</v>
+      </c>
+      <c r="D31" t="s">
+        <v>2</v>
       </c>
       <c r="E31" t="s">
         <v>2</v>
       </c>
       <c r="F31">
-        <v>1</v>
-      </c>
-      <c r="G31">
-        <v>41.421600000000005</v>
+        <v>0</v>
+      </c>
+      <c r="G31" t="s">
+        <v>2</v>
       </c>
       <c r="H31" t="s">
         <v>2</v>
       </c>
       <c r="I31">
-        <v>1</v>
-      </c>
-      <c r="J31" t="s">
-        <v>2</v>
-      </c>
-      <c r="K31" t="s">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>-430.83333333333331</v>
+      </c>
+      <c r="K31">
+        <v>2.2546248764114472</v>
       </c>
       <c r="L31">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C32" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="D32">
-        <v>295.14999999999998</v>
+        <v>264.14999999999998</v>
       </c>
       <c r="E32" t="s">
         <v>2</v>
@@ -1725,14 +1806,14 @@
       <c r="F32">
         <v>1</v>
       </c>
-      <c r="G32">
-        <v>1.29704</v>
+      <c r="G32" t="s">
+        <v>2</v>
       </c>
       <c r="H32" t="s">
         <v>2</v>
       </c>
       <c r="I32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J32" t="s">
         <v>2</v>
@@ -1746,13 +1827,13 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C33" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="D33">
-        <v>412.15</v>
+        <v>377.15</v>
       </c>
       <c r="E33" t="s">
         <v>2</v>
@@ -1761,7 +1842,7 @@
         <v>1</v>
       </c>
       <c r="G33">
-        <v>39.329600000000006</v>
+        <v>15.8992</v>
       </c>
       <c r="H33" t="s">
         <v>2</v>
@@ -1781,10 +1862,10 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C34" t="s">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="D34" t="s">
         <v>2</v>
@@ -1805,33 +1886,33 @@
         <v>0</v>
       </c>
       <c r="J34">
-        <v>-442</v>
-      </c>
-      <c r="K34" t="s">
-        <v>2</v>
+        <v>-256.83333333333331</v>
+      </c>
+      <c r="K34">
+        <v>9.6738479072876338</v>
       </c>
       <c r="L34">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C35" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D35">
-        <v>459.61</v>
+        <v>653.01</v>
       </c>
       <c r="E35">
-        <v>61.461721420734726</v>
+        <v>56.766532393656014</v>
       </c>
       <c r="F35">
         <v>2</v>
       </c>
       <c r="G35">
-        <v>66.58</v>
+        <v>20.49</v>
       </c>
       <c r="H35" t="s">
         <v>2</v>
@@ -1840,21 +1921,21 @@
         <v>1</v>
       </c>
       <c r="J35">
-        <v>-487.5</v>
+        <v>-274.8</v>
       </c>
       <c r="K35">
-        <v>17.677669529663689</v>
+        <v>2.4331050121192805</v>
       </c>
       <c r="L35">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C36" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="D36" t="s">
         <v>2</v>
@@ -1875,47 +1956,292 @@
         <v>0</v>
       </c>
       <c r="J36">
-        <v>-395</v>
-      </c>
-      <c r="K36" t="s">
-        <v>2</v>
+        <v>-199.13333333333333</v>
+      </c>
+      <c r="K36">
+        <v>7.9122268251948746</v>
       </c>
       <c r="L36">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>7</v>
+      </c>
+      <c r="C37" t="s">
+        <v>8</v>
+      </c>
+      <c r="D37">
+        <v>683</v>
+      </c>
+      <c r="E37" t="s">
+        <v>2</v>
+      </c>
+      <c r="F37">
+        <v>1</v>
+      </c>
+      <c r="G37">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="H37" t="s">
+        <v>2</v>
+      </c>
+      <c r="I37">
+        <v>1</v>
+      </c>
+      <c r="J37">
+        <v>-330.4</v>
+      </c>
+      <c r="K37">
+        <v>1.4071247279470325</v>
+      </c>
+      <c r="L37">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>58</v>
+      </c>
+      <c r="C38" t="s">
+        <v>72</v>
+      </c>
+      <c r="D38">
+        <v>376.15</v>
+      </c>
+      <c r="E38" t="s">
+        <v>2</v>
+      </c>
+      <c r="F38">
+        <v>1</v>
+      </c>
+      <c r="G38">
+        <v>41.421600000000005</v>
+      </c>
+      <c r="H38" t="s">
+        <v>2</v>
+      </c>
+      <c r="I38">
+        <v>1</v>
+      </c>
+      <c r="J38" t="s">
+        <v>2</v>
+      </c>
+      <c r="K38" t="s">
+        <v>2</v>
+      </c>
+      <c r="L38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>59</v>
+      </c>
+      <c r="C39" t="s">
+        <v>73</v>
+      </c>
+      <c r="D39">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="E39" t="s">
+        <v>2</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39">
+        <v>1.29704</v>
+      </c>
+      <c r="H39" t="s">
+        <v>2</v>
+      </c>
+      <c r="I39">
+        <v>1</v>
+      </c>
+      <c r="J39" t="s">
+        <v>2</v>
+      </c>
+      <c r="K39" t="s">
+        <v>2</v>
+      </c>
+      <c r="L39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>60</v>
+      </c>
+      <c r="C40" t="s">
+        <v>74</v>
+      </c>
+      <c r="D40">
+        <v>412.15</v>
+      </c>
+      <c r="E40" t="s">
+        <v>2</v>
+      </c>
+      <c r="F40">
+        <v>1</v>
+      </c>
+      <c r="G40">
+        <v>39.329600000000006</v>
+      </c>
+      <c r="H40" t="s">
+        <v>2</v>
+      </c>
+      <c r="I40">
+        <v>1</v>
+      </c>
+      <c r="J40" t="s">
+        <v>2</v>
+      </c>
+      <c r="K40" t="s">
+        <v>2</v>
+      </c>
+      <c r="L40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>61</v>
+      </c>
+      <c r="C41" t="s">
+        <v>75</v>
+      </c>
+      <c r="D41" t="s">
+        <v>2</v>
+      </c>
+      <c r="E41" t="s">
+        <v>2</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41" t="s">
+        <v>2</v>
+      </c>
+      <c r="H41" t="s">
+        <v>2</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>-442</v>
+      </c>
+      <c r="K41" t="s">
+        <v>2</v>
+      </c>
+      <c r="L41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42" t="s">
+        <v>22</v>
+      </c>
+      <c r="D42">
+        <v>459.61</v>
+      </c>
+      <c r="E42">
+        <v>61.461721420734726</v>
+      </c>
+      <c r="F42">
+        <v>2</v>
+      </c>
+      <c r="G42">
+        <v>66.58</v>
+      </c>
+      <c r="H42" t="s">
+        <v>2</v>
+      </c>
+      <c r="I42">
+        <v>1</v>
+      </c>
+      <c r="J42">
+        <v>-487.5</v>
+      </c>
+      <c r="K42">
+        <v>17.677669529663689</v>
+      </c>
+      <c r="L42">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>62</v>
+      </c>
+      <c r="C43" t="s">
+        <v>76</v>
+      </c>
+      <c r="D43" t="s">
+        <v>2</v>
+      </c>
+      <c r="E43" t="s">
+        <v>2</v>
+      </c>
+      <c r="F43">
+        <v>0</v>
+      </c>
+      <c r="G43" t="s">
+        <v>2</v>
+      </c>
+      <c r="H43" t="s">
+        <v>2</v>
+      </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+      <c r="J43">
+        <v>-395</v>
+      </c>
+      <c r="K43" t="s">
+        <v>2</v>
+      </c>
+      <c r="L43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>41</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C44" t="s">
         <v>42</v>
       </c>
-      <c r="D37">
+      <c r="D44">
         <v>153.26</v>
       </c>
-      <c r="E37">
+      <c r="E44">
         <v>3.6390932936653244</v>
       </c>
-      <c r="F37">
+      <c r="F44">
         <v>5</v>
       </c>
-      <c r="G37">
+      <c r="G44">
         <v>6.5419999999999998</v>
       </c>
-      <c r="H37">
+      <c r="H44">
         <v>2.8284271247458787E-3</v>
       </c>
-      <c r="I37">
-        <v>2</v>
-      </c>
-      <c r="J37">
+      <c r="I44">
+        <v>2</v>
+      </c>
+      <c r="J44">
         <v>-27.2</v>
       </c>
-      <c r="K37">
+      <c r="K44">
         <v>4.9497474683058327</v>
       </c>
-      <c r="L37">
+      <c r="L44">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added associated elements. Made results worse.
</commit_message>
<xml_diff>
--- a/MTGPR_train.xlsx
+++ b/MTGPR_train.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB52E98-A14D-4C1B-833B-67AFECD6D4C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D0664E-13FA-4515-B364-52EF6EEF08F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="113">
   <si>
     <t>tetrabutylammonium bromide</t>
   </si>
@@ -312,6 +312,72 @@
   </si>
   <si>
     <t>CNN</t>
+  </si>
+  <si>
+    <t>boron</t>
+  </si>
+  <si>
+    <t>[B]</t>
+  </si>
+  <si>
+    <t>calcium</t>
+  </si>
+  <si>
+    <t>[Ca]</t>
+  </si>
+  <si>
+    <t>carbon</t>
+  </si>
+  <si>
+    <t>[C]</t>
+  </si>
+  <si>
+    <t>dichlorine</t>
+  </si>
+  <si>
+    <t>ClCl</t>
+  </si>
+  <si>
+    <t>dihydrogen</t>
+  </si>
+  <si>
+    <t>[HH]</t>
+  </si>
+  <si>
+    <t>dinitrogen</t>
+  </si>
+  <si>
+    <t>N#N</t>
+  </si>
+  <si>
+    <t>dioxygen</t>
+  </si>
+  <si>
+    <t>O=O</t>
+  </si>
+  <si>
+    <t>lithium</t>
+  </si>
+  <si>
+    <t>[Li]</t>
+  </si>
+  <si>
+    <t>potassium</t>
+  </si>
+  <si>
+    <t>[K]</t>
+  </si>
+  <si>
+    <t>sodium</t>
+  </si>
+  <si>
+    <t>[Na]</t>
+  </si>
+  <si>
+    <t>sulfur</t>
+  </si>
+  <si>
+    <t>[S]</t>
   </si>
 </sst>
 </file>
@@ -719,7 +785,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -847,31 +913,31 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="C5" t="s">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="D5">
-        <v>160.91</v>
-      </c>
-      <c r="E5">
-        <v>0.52844110362461461</v>
+        <v>2349.15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>2</v>
       </c>
       <c r="F5">
-        <v>5</v>
-      </c>
-      <c r="G5" t="s">
-        <v>2</v>
-      </c>
-      <c r="H5" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G5">
+        <v>50.133333333333333</v>
+      </c>
+      <c r="H5">
+        <v>0.1154700538379268</v>
       </c>
       <c r="I5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J5" s="2">
-        <v>-5.8</v>
+        <v>0</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>2</v>
@@ -882,101 +948,101 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D6">
-        <v>245.31</v>
+        <v>160.91</v>
       </c>
       <c r="E6">
-        <v>1.4142135623718088E-2</v>
+        <v>0.52844110362461461</v>
       </c>
       <c r="F6">
-        <v>2</v>
-      </c>
-      <c r="G6">
-        <v>8.1095000000000006</v>
-      </c>
-      <c r="H6">
-        <v>7.0710678118615568E-4</v>
+        <v>5</v>
+      </c>
+      <c r="G6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H6" t="s">
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J6" s="2">
-        <v>296.91750000000002</v>
-      </c>
-      <c r="K6" s="2">
-        <v>22.637415009963771</v>
+        <v>-5.8</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L6">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>93</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>94</v>
       </c>
       <c r="D7">
-        <v>179.32</v>
-      </c>
-      <c r="E7">
-        <v>1.3349157276772183</v>
+        <v>1115.1500000000001</v>
+      </c>
+      <c r="E7" t="s">
+        <v>2</v>
       </c>
       <c r="F7">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G7">
-        <v>5.9405000000000001</v>
+        <v>8.5399999999999991</v>
       </c>
       <c r="H7">
-        <v>7.0710678118615568E-4</v>
+        <v>0</v>
       </c>
       <c r="I7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J7" s="2">
-        <v>-21.4</v>
-      </c>
-      <c r="K7" s="2">
-        <v>3.3941125496954587</v>
+        <v>0</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L7">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="C8" t="s">
-        <v>84</v>
-      </c>
-      <c r="D8">
-        <v>215.97499999999999</v>
-      </c>
-      <c r="E8">
-        <v>3.5355339059335411E-2</v>
+        <v>96</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>2</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G8">
-        <v>10.071300000000001</v>
+        <v>117</v>
       </c>
       <c r="H8">
-        <v>1.838477631084507E-3</v>
+        <v>0</v>
       </c>
       <c r="I8">
         <v>2</v>
       </c>
       <c r="J8" s="2">
-        <v>48.3</v>
+        <v>0</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>2</v>
@@ -987,83 +1053,83 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C9" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="D9">
-        <v>263.84999999999997</v>
-      </c>
-      <c r="E9" t="s">
-        <v>2</v>
+        <v>245.31</v>
+      </c>
+      <c r="E9">
+        <v>1.4142135623718088E-2</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>14.65</v>
-      </c>
-      <c r="H9" t="s">
-        <v>2</v>
+        <v>8.1095000000000006</v>
+      </c>
+      <c r="H9">
+        <v>7.0710678118615568E-4</v>
       </c>
       <c r="I9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="2">
-        <v>9.08</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>2</v>
+        <v>296.91750000000002</v>
+      </c>
+      <c r="K9" s="2">
+        <v>22.637415009963771</v>
       </c>
       <c r="L9">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>25</v>
+        <v>97</v>
       </c>
       <c r="C10" t="s">
-        <v>26</v>
+        <v>98</v>
       </c>
       <c r="D10">
-        <v>95.1</v>
-      </c>
-      <c r="E10">
-        <v>8.3438600180012585</v>
+        <v>171.64999999999998</v>
+      </c>
+      <c r="E10" t="s">
+        <v>2</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10">
-        <v>2.8133333333333339</v>
+        <v>6.4030000000000005</v>
       </c>
       <c r="H10">
-        <v>3.7846179904097832E-2</v>
+        <v>4.2426406871188182E-3</v>
       </c>
       <c r="I10">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J10" s="2">
-        <v>-84.15666666666668</v>
-      </c>
-      <c r="K10" s="2">
-        <v>0.45566800780100331</v>
+        <v>0</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L10">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>44</v>
+        <v>99</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="D11">
-        <v>155</v>
+        <v>14.009999999999991</v>
       </c>
       <c r="E11" t="s">
         <v>2</v>
@@ -1071,17 +1137,17 @@
       <c r="F11">
         <v>1</v>
       </c>
-      <c r="G11" t="s">
-        <v>2</v>
-      </c>
-      <c r="H11" t="s">
-        <v>2</v>
+      <c r="G11">
+        <v>0.11849999999999999</v>
+      </c>
+      <c r="H11">
+        <v>2.1213203435596346E-3</v>
       </c>
       <c r="I11">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J11" s="2">
-        <v>-95.5</v>
+        <v>0</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>2</v>
@@ -1092,101 +1158,101 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="D12">
-        <v>134.76249999999999</v>
+        <v>179.32</v>
       </c>
       <c r="E12">
-        <v>2.4581073342445094</v>
+        <v>1.3349157276772183</v>
       </c>
       <c r="F12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G12">
-        <v>4.4510000000000005</v>
+        <v>5.9405000000000001</v>
       </c>
       <c r="H12">
-        <v>1.4142135623729393E-3</v>
+        <v>7.0710678118615568E-4</v>
       </c>
       <c r="I12">
         <v>2</v>
       </c>
       <c r="J12" s="2">
-        <v>-137</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>2</v>
+        <v>-21.4</v>
+      </c>
+      <c r="K12" s="2">
+        <v>3.3941125496954587</v>
       </c>
       <c r="L12">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>46</v>
+        <v>83</v>
       </c>
       <c r="C13" t="s">
-        <v>47</v>
+        <v>84</v>
       </c>
       <c r="D13">
-        <v>162.17500000000001</v>
+        <v>215.97499999999999</v>
       </c>
       <c r="E13">
-        <v>0.17677669529663689</v>
+        <v>3.5355339059335411E-2</v>
       </c>
       <c r="F13">
         <v>2</v>
       </c>
-      <c r="G13" t="s">
-        <v>2</v>
-      </c>
-      <c r="H13" t="s">
-        <v>2</v>
+      <c r="G13">
+        <v>10.071300000000001</v>
+      </c>
+      <c r="H13">
+        <v>1.838477631084507E-3</v>
       </c>
       <c r="I13">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J13" s="2">
-        <v>-37.866666666666667</v>
-      </c>
-      <c r="K13" s="2">
-        <v>2.4906491790963527</v>
+        <v>48.3</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L13">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="D14">
-        <v>274.93333333333334</v>
-      </c>
-      <c r="E14">
-        <v>0.25658007197234717</v>
+        <v>63.049999999999983</v>
+      </c>
+      <c r="E14" t="s">
+        <v>2</v>
       </c>
       <c r="F14">
-        <v>3</v>
-      </c>
-      <c r="G14" t="s">
-        <v>2</v>
-      </c>
-      <c r="H14" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G14">
+        <v>0.71499999999999997</v>
+      </c>
+      <c r="H14">
+        <v>7.0710678118654814E-3</v>
       </c>
       <c r="I14">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J14" s="2">
-        <v>50.63</v>
+        <v>0</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>2</v>
@@ -1197,22 +1263,22 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="C15" t="s">
-        <v>30</v>
+        <v>86</v>
       </c>
       <c r="D15">
-        <v>89.72</v>
-      </c>
-      <c r="E15">
-        <v>2.2642879675518288</v>
+        <v>263.84999999999997</v>
+      </c>
+      <c r="E15" t="s">
+        <v>2</v>
       </c>
       <c r="F15">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G15">
-        <v>0.93920000000000003</v>
+        <v>14.65</v>
       </c>
       <c r="H15" t="s">
         <v>2</v>
@@ -1221,24 +1287,24 @@
         <v>1</v>
       </c>
       <c r="J15" s="2">
-        <v>-74.444000000000003</v>
-      </c>
-      <c r="K15" s="2">
-        <v>0.60492148250826439</v>
+        <v>9.08</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L15">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>31</v>
+        <v>103</v>
       </c>
       <c r="C16" t="s">
-        <v>32</v>
+        <v>104</v>
       </c>
       <c r="D16">
-        <v>179.5</v>
+        <v>327.95</v>
       </c>
       <c r="E16" t="s">
         <v>2</v>
@@ -1247,16 +1313,16 @@
         <v>1</v>
       </c>
       <c r="G16">
-        <v>5.98</v>
-      </c>
-      <c r="H16" t="s">
-        <v>2</v>
+        <v>0.442</v>
+      </c>
+      <c r="H16">
+        <v>2.8284271247461927E-3</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J16" s="2">
-        <v>-60.6</v>
+        <v>0</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>2</v>
@@ -1267,171 +1333,171 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="C17" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="D17">
-        <v>178.01666666666665</v>
+        <v>95.1</v>
       </c>
       <c r="E17">
-        <v>3.4822167269331912</v>
+        <v>8.3438600180012585</v>
       </c>
       <c r="F17">
+        <v>2</v>
+      </c>
+      <c r="G17">
+        <v>2.8133333333333339</v>
+      </c>
+      <c r="H17">
+        <v>3.7846179904097832E-2</v>
+      </c>
+      <c r="I17">
         <v>3</v>
       </c>
-      <c r="G17">
-        <v>6.4254999999999995</v>
-      </c>
-      <c r="H17">
-        <v>7.778174593052108E-3</v>
-      </c>
-      <c r="I17">
-        <v>2</v>
-      </c>
       <c r="J17" s="2">
-        <v>-102.4</v>
-      </c>
-      <c r="K17" s="2" t="s">
-        <v>2</v>
+        <v>-84.15666666666668</v>
+      </c>
+      <c r="K17" s="2">
+        <v>0.45566800780100331</v>
       </c>
       <c r="L17">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="D18">
-        <v>207.39999999999998</v>
-      </c>
-      <c r="E18">
-        <v>0.98994949366117058</v>
+        <v>155</v>
+      </c>
+      <c r="E18" t="s">
+        <v>2</v>
       </c>
       <c r="F18">
-        <v>2</v>
-      </c>
-      <c r="G18">
-        <v>9.1199999999999992</v>
+        <v>1</v>
+      </c>
+      <c r="G18" t="s">
+        <v>2</v>
       </c>
       <c r="H18" t="s">
         <v>2</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" s="2">
-        <v>-12.8</v>
-      </c>
-      <c r="K18" s="2">
-        <v>1.1313708498984758</v>
+        <v>-95.5</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L18">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="D19">
-        <v>179.93333333333331</v>
+        <v>134.76249999999999</v>
       </c>
       <c r="E19">
-        <v>0.20207259421638213</v>
+        <v>2.4581073342445094</v>
       </c>
       <c r="F19">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G19">
-        <v>6.1319999999999997</v>
+        <v>4.4510000000000005</v>
       </c>
       <c r="H19">
-        <v>2.8284271247465066E-3</v>
+        <v>1.4142135623729393E-3</v>
       </c>
       <c r="I19">
         <v>2</v>
       </c>
       <c r="J19" s="2">
-        <v>-17.850000000000001</v>
-      </c>
-      <c r="K19" s="2">
-        <v>7.9903066274079748</v>
+        <v>-137</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L19">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>89</v>
+        <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>90</v>
+        <v>47</v>
       </c>
       <c r="D20">
-        <v>220.79500000000002</v>
+        <v>162.17500000000001</v>
       </c>
       <c r="E20">
-        <v>7.0710678118791415E-3</v>
+        <v>0.17677669529663689</v>
       </c>
       <c r="F20">
         <v>2</v>
       </c>
-      <c r="G20">
-        <v>10.419</v>
-      </c>
-      <c r="H20">
-        <v>1.4142135623735675E-3</v>
+      <c r="G20" t="s">
+        <v>2</v>
+      </c>
+      <c r="H20" t="s">
+        <v>2</v>
       </c>
       <c r="I20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J20" s="2">
-        <v>54.14</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>2</v>
+        <v>-37.866666666666667</v>
+      </c>
+      <c r="K20" s="2">
+        <v>2.4906491790963527</v>
       </c>
       <c r="L20">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="C21" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="D21">
-        <v>180</v>
-      </c>
-      <c r="E21" t="s">
-        <v>2</v>
+        <v>274.93333333333334</v>
+      </c>
+      <c r="E21">
+        <v>0.25658007197234717</v>
       </c>
       <c r="F21">
-        <v>1</v>
-      </c>
-      <c r="G21">
-        <v>5.03</v>
+        <v>3</v>
+      </c>
+      <c r="G21" t="s">
+        <v>2</v>
       </c>
       <c r="H21" t="s">
         <v>2</v>
       </c>
       <c r="I21">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J21">
-        <v>15.5</v>
+        <v>50.63</v>
       </c>
       <c r="K21" t="s">
         <v>2</v>
@@ -1442,13 +1508,13 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>39</v>
+        <v>105</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>106</v>
       </c>
       <c r="D22">
-        <v>190.15</v>
+        <v>453.68999999999994</v>
       </c>
       <c r="E22" t="s">
         <v>2</v>
@@ -1457,68 +1523,68 @@
         <v>1</v>
       </c>
       <c r="G22">
-        <v>10.856400000000001</v>
+        <v>3</v>
       </c>
       <c r="H22">
-        <v>0.20040928122220297</v>
+        <v>0</v>
       </c>
       <c r="I22">
         <v>3</v>
       </c>
       <c r="J22">
-        <v>-119.75</v>
-      </c>
-      <c r="K22">
-        <v>25.809397513308983</v>
+        <v>0</v>
+      </c>
+      <c r="K22" t="s">
+        <v>2</v>
       </c>
       <c r="L22">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="C23" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="D23">
-        <v>395.07499999999999</v>
+        <v>89.72</v>
       </c>
       <c r="E23">
-        <v>0.10606601717796604</v>
+        <v>2.2642879675518288</v>
       </c>
       <c r="F23">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G23">
-        <v>15.8154</v>
-      </c>
-      <c r="H23">
-        <v>0.47319585797003511</v>
+        <v>0.93920000000000003</v>
+      </c>
+      <c r="H23" t="s">
+        <v>2</v>
       </c>
       <c r="I23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J23">
-        <v>-477.65</v>
+        <v>-74.444000000000003</v>
       </c>
       <c r="K23">
-        <v>88.600479682674319</v>
+        <v>0.60492148250826439</v>
       </c>
       <c r="L23">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>49</v>
+        <v>31</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="D24">
-        <v>314.14999999999998</v>
+        <v>179.5</v>
       </c>
       <c r="E24" t="s">
         <v>2</v>
@@ -1527,7 +1593,7 @@
         <v>1</v>
       </c>
       <c r="G24">
-        <v>20.501600000000003</v>
+        <v>5.98</v>
       </c>
       <c r="H24" t="s">
         <v>2</v>
@@ -1536,164 +1602,164 @@
         <v>1</v>
       </c>
       <c r="J24">
-        <v>-549.4</v>
-      </c>
-      <c r="K24">
-        <v>21.778888860545631</v>
+        <v>-60.6</v>
+      </c>
+      <c r="K24" t="s">
+        <v>2</v>
       </c>
       <c r="L24">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C25" t="s">
+        <v>34</v>
+      </c>
+      <c r="D25">
+        <v>178.01666666666665</v>
+      </c>
+      <c r="E25">
+        <v>3.4822167269331912</v>
+      </c>
+      <c r="F25">
         <v>3</v>
       </c>
-      <c r="C25" t="s">
-        <v>4</v>
-      </c>
-      <c r="D25">
-        <v>419.15</v>
-      </c>
-      <c r="E25" t="s">
-        <v>2</v>
-      </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
       <c r="G25">
-        <v>9.6231999999999989</v>
-      </c>
-      <c r="H25" t="s">
-        <v>2</v>
+        <v>6.4254999999999995</v>
+      </c>
+      <c r="H25">
+        <v>7.778174593052108E-3</v>
       </c>
       <c r="I25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J25">
-        <v>-479.3</v>
-      </c>
-      <c r="K25">
-        <v>27.294321753800752</v>
+        <v>-102.4</v>
+      </c>
+      <c r="K25" t="s">
+        <v>2</v>
       </c>
       <c r="L25">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="C26" t="s">
-        <v>6</v>
+        <v>36</v>
       </c>
       <c r="D26">
-        <v>389.9666666666667</v>
+        <v>207.39999999999998</v>
       </c>
       <c r="E26">
-        <v>1.9857828011475314</v>
+        <v>0.98994949366117058</v>
       </c>
       <c r="F26">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G26">
-        <v>14.95</v>
-      </c>
-      <c r="H26">
-        <v>0.91923881554251108</v>
+        <v>9.1199999999999992</v>
+      </c>
+      <c r="H26" t="s">
+        <v>2</v>
       </c>
       <c r="I26">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J26">
-        <v>-600.20000000000005</v>
-      </c>
-      <c r="K26" t="s">
-        <v>2</v>
+        <v>-12.8</v>
+      </c>
+      <c r="K26">
+        <v>1.1313708498984758</v>
       </c>
       <c r="L26">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="C27" t="s">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="D27">
-        <v>502.2</v>
-      </c>
-      <c r="E27" t="s">
-        <v>2</v>
+        <v>179.93333333333331</v>
+      </c>
+      <c r="E27">
+        <v>0.20207259421638213</v>
       </c>
       <c r="F27">
-        <v>1</v>
-      </c>
-      <c r="G27" t="s">
-        <v>2</v>
-      </c>
-      <c r="H27" t="s">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="G27">
+        <v>6.1319999999999997</v>
+      </c>
+      <c r="H27">
+        <v>2.8284271247465066E-3</v>
       </c>
       <c r="I27">
-        <v>0</v>
-      </c>
-      <c r="J27" t="s">
-        <v>2</v>
-      </c>
-      <c r="K27" t="s">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="J27">
+        <v>-17.850000000000001</v>
+      </c>
+      <c r="K27">
+        <v>7.9903066274079748</v>
       </c>
       <c r="L27">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>15</v>
+        <v>89</v>
       </c>
       <c r="C28" t="s">
-        <v>16</v>
+        <v>90</v>
       </c>
       <c r="D28">
-        <v>447</v>
-      </c>
-      <c r="E28" t="s">
-        <v>2</v>
+        <v>220.79500000000002</v>
+      </c>
+      <c r="E28">
+        <v>7.0710678118791415E-3</v>
       </c>
       <c r="F28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G28">
-        <v>20.3</v>
-      </c>
-      <c r="H28" t="s">
-        <v>2</v>
+        <v>10.419</v>
+      </c>
+      <c r="H28">
+        <v>1.4142135623735675E-3</v>
       </c>
       <c r="I28">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J28">
-        <v>-363.45</v>
-      </c>
-      <c r="K28">
-        <v>15.700212312789498</v>
+        <v>54.14</v>
+      </c>
+      <c r="K28" t="s">
+        <v>2</v>
       </c>
       <c r="L28">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>17</v>
+        <v>107</v>
       </c>
       <c r="C29" t="s">
-        <v>18</v>
+        <v>108</v>
       </c>
       <c r="D29">
-        <v>526.78</v>
+        <v>336.53</v>
       </c>
       <c r="E29" t="s">
         <v>2</v>
@@ -1702,103 +1768,103 @@
         <v>1</v>
       </c>
       <c r="G29">
-        <v>51.24</v>
-      </c>
-      <c r="H29" t="s">
-        <v>2</v>
+        <v>2.327</v>
+      </c>
+      <c r="H29">
+        <v>5.1961524227065728E-3</v>
       </c>
       <c r="I29">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J29">
-        <v>-396.29999999999995</v>
-      </c>
-      <c r="K29">
-        <v>18.966988866624746</v>
+        <v>0</v>
+      </c>
+      <c r="K29" t="s">
+        <v>2</v>
       </c>
       <c r="L29">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
-      </c>
-      <c r="D30" t="s">
-        <v>2</v>
+        <v>64</v>
+      </c>
+      <c r="D30">
+        <v>180</v>
       </c>
       <c r="E30" t="s">
         <v>2</v>
       </c>
       <c r="F30">
-        <v>0</v>
-      </c>
-      <c r="G30" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G30">
+        <v>5.03</v>
       </c>
       <c r="H30" t="s">
         <v>2</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J30">
-        <v>-316.17500000000001</v>
-      </c>
-      <c r="K30">
-        <v>12.790198069876276</v>
+        <v>15.5</v>
+      </c>
+      <c r="K30" t="s">
+        <v>2</v>
       </c>
       <c r="L30">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
-      </c>
-      <c r="D31" t="s">
-        <v>2</v>
+        <v>40</v>
+      </c>
+      <c r="D31">
+        <v>190.15</v>
       </c>
       <c r="E31" t="s">
         <v>2</v>
       </c>
       <c r="F31">
-        <v>0</v>
-      </c>
-      <c r="G31" t="s">
-        <v>2</v>
-      </c>
-      <c r="H31" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G31">
+        <v>10.856400000000001</v>
+      </c>
+      <c r="H31">
+        <v>0.20040928122220297</v>
       </c>
       <c r="I31">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J31">
-        <v>-430.83333333333331</v>
+        <v>-119.75</v>
       </c>
       <c r="K31">
-        <v>2.2546248764114472</v>
+        <v>25.809397513308983</v>
       </c>
       <c r="L31">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>54</v>
+        <v>109</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>110</v>
       </c>
       <c r="D32">
-        <v>264.14999999999998</v>
+        <v>370.87</v>
       </c>
       <c r="E32" t="s">
         <v>2</v>
@@ -1806,34 +1872,34 @@
       <c r="F32">
         <v>1</v>
       </c>
-      <c r="G32" t="s">
-        <v>2</v>
-      </c>
-      <c r="H32" t="s">
-        <v>2</v>
+      <c r="G32">
+        <v>2.6</v>
+      </c>
+      <c r="H32">
+        <v>0</v>
       </c>
       <c r="I32">
-        <v>0</v>
-      </c>
-      <c r="J32" t="s">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="J32">
+        <v>0</v>
       </c>
       <c r="K32" t="s">
         <v>2</v>
       </c>
       <c r="L32">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>111</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="D33">
-        <v>377.15</v>
+        <v>368.45</v>
       </c>
       <c r="E33" t="s">
         <v>2</v>
@@ -1842,77 +1908,77 @@
         <v>1</v>
       </c>
       <c r="G33">
-        <v>15.8992</v>
-      </c>
-      <c r="H33" t="s">
-        <v>2</v>
+        <v>1.7256666666666665</v>
+      </c>
+      <c r="H33">
+        <v>5.1316014394469037E-3</v>
       </c>
       <c r="I33">
-        <v>1</v>
-      </c>
-      <c r="J33" t="s">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="J33">
+        <v>0</v>
       </c>
       <c r="K33" t="s">
         <v>2</v>
       </c>
       <c r="L33">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>56</v>
+        <v>0</v>
       </c>
       <c r="C34" t="s">
-        <v>70</v>
-      </c>
-      <c r="D34" t="s">
-        <v>2</v>
-      </c>
-      <c r="E34" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D34">
+        <v>395.07499999999999</v>
+      </c>
+      <c r="E34">
+        <v>0.10606601717796604</v>
       </c>
       <c r="F34">
-        <v>0</v>
-      </c>
-      <c r="G34" t="s">
-        <v>2</v>
-      </c>
-      <c r="H34" t="s">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="G34">
+        <v>15.8154</v>
+      </c>
+      <c r="H34">
+        <v>0.47319585797003511</v>
       </c>
       <c r="I34">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J34">
-        <v>-256.83333333333331</v>
+        <v>-477.65</v>
       </c>
       <c r="K34">
-        <v>9.6738479072876338</v>
+        <v>88.600479682674319</v>
       </c>
       <c r="L34">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>19</v>
+        <v>49</v>
       </c>
       <c r="C35" t="s">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="D35">
-        <v>653.01</v>
-      </c>
-      <c r="E35">
-        <v>56.766532393656014</v>
+        <v>314.14999999999998</v>
+      </c>
+      <c r="E35" t="s">
+        <v>2</v>
       </c>
       <c r="F35">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G35">
-        <v>20.49</v>
+        <v>20.501600000000003</v>
       </c>
       <c r="H35" t="s">
         <v>2</v>
@@ -1921,94 +1987,94 @@
         <v>1</v>
       </c>
       <c r="J35">
-        <v>-274.8</v>
+        <v>-549.4</v>
       </c>
       <c r="K35">
-        <v>2.4331050121192805</v>
+        <v>21.778888860545631</v>
       </c>
       <c r="L35">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>57</v>
+        <v>3</v>
       </c>
       <c r="C36" t="s">
-        <v>71</v>
-      </c>
-      <c r="D36" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="D36">
+        <v>419.15</v>
       </c>
       <c r="E36" t="s">
         <v>2</v>
       </c>
       <c r="F36">
-        <v>0</v>
-      </c>
-      <c r="G36" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G36">
+        <v>9.6231999999999989</v>
       </c>
       <c r="H36" t="s">
         <v>2</v>
       </c>
       <c r="I36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J36">
-        <v>-199.13333333333333</v>
+        <v>-479.3</v>
       </c>
       <c r="K36">
-        <v>7.9122268251948746</v>
+        <v>27.294321753800752</v>
       </c>
       <c r="L36">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C37" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D37">
-        <v>683</v>
-      </c>
-      <c r="E37" t="s">
-        <v>2</v>
+        <v>389.9666666666667</v>
+      </c>
+      <c r="E37">
+        <v>1.9857828011475314</v>
       </c>
       <c r="F37">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G37">
-        <v>37.200000000000003</v>
-      </c>
-      <c r="H37" t="s">
-        <v>2</v>
+        <v>14.95</v>
+      </c>
+      <c r="H37">
+        <v>0.91923881554251108</v>
       </c>
       <c r="I37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J37">
-        <v>-330.4</v>
-      </c>
-      <c r="K37">
-        <v>1.4071247279470325</v>
+        <v>-600.20000000000005</v>
+      </c>
+      <c r="K37" t="s">
+        <v>2</v>
       </c>
       <c r="L37">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="D38">
-        <v>376.15</v>
+        <v>502.2</v>
       </c>
       <c r="E38" t="s">
         <v>2</v>
@@ -2016,14 +2082,14 @@
       <c r="F38">
         <v>1</v>
       </c>
-      <c r="G38">
-        <v>41.421600000000005</v>
+      <c r="G38" t="s">
+        <v>2</v>
       </c>
       <c r="H38" t="s">
         <v>2</v>
       </c>
       <c r="I38">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J38" t="s">
         <v>2</v>
@@ -2037,13 +2103,13 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="C39" t="s">
-        <v>73</v>
+        <v>16</v>
       </c>
       <c r="D39">
-        <v>295.14999999999998</v>
+        <v>447</v>
       </c>
       <c r="E39" t="s">
         <v>2</v>
@@ -2052,7 +2118,7 @@
         <v>1</v>
       </c>
       <c r="G39">
-        <v>1.29704</v>
+        <v>20.3</v>
       </c>
       <c r="H39" t="s">
         <v>2</v>
@@ -2060,25 +2126,25 @@
       <c r="I39">
         <v>1</v>
       </c>
-      <c r="J39" t="s">
-        <v>2</v>
-      </c>
-      <c r="K39" t="s">
-        <v>2</v>
+      <c r="J39">
+        <v>-363.45</v>
+      </c>
+      <c r="K39">
+        <v>15.700212312789498</v>
       </c>
       <c r="L39">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="C40" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="D40">
-        <v>412.15</v>
+        <v>526.78</v>
       </c>
       <c r="E40" t="s">
         <v>2</v>
@@ -2087,7 +2153,7 @@
         <v>1</v>
       </c>
       <c r="G40">
-        <v>39.329600000000006</v>
+        <v>51.24</v>
       </c>
       <c r="H40" t="s">
         <v>2</v>
@@ -2095,22 +2161,22 @@
       <c r="I40">
         <v>1</v>
       </c>
-      <c r="J40" t="s">
-        <v>2</v>
-      </c>
-      <c r="K40" t="s">
-        <v>2</v>
+      <c r="J40">
+        <v>-396.29999999999995</v>
+      </c>
+      <c r="K40">
+        <v>18.966988866624746</v>
       </c>
       <c r="L40">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C41" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="D41" t="s">
         <v>2</v>
@@ -2131,65 +2197,65 @@
         <v>0</v>
       </c>
       <c r="J41">
-        <v>-442</v>
-      </c>
-      <c r="K41" t="s">
-        <v>2</v>
+        <v>-316.17500000000001</v>
+      </c>
+      <c r="K41">
+        <v>12.790198069876276</v>
       </c>
       <c r="L41">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="C42" t="s">
-        <v>22</v>
-      </c>
-      <c r="D42">
-        <v>459.61</v>
-      </c>
-      <c r="E42">
-        <v>61.461721420734726</v>
+        <v>67</v>
+      </c>
+      <c r="D42" t="s">
+        <v>2</v>
+      </c>
+      <c r="E42" t="s">
+        <v>2</v>
       </c>
       <c r="F42">
-        <v>2</v>
-      </c>
-      <c r="G42">
-        <v>66.58</v>
+        <v>0</v>
+      </c>
+      <c r="G42" t="s">
+        <v>2</v>
       </c>
       <c r="H42" t="s">
         <v>2</v>
       </c>
       <c r="I42">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J42">
-        <v>-487.5</v>
+        <v>-430.83333333333331</v>
       </c>
       <c r="K42">
-        <v>17.677669529663689</v>
+        <v>2.2546248764114472</v>
       </c>
       <c r="L42">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="C43" t="s">
-        <v>76</v>
-      </c>
-      <c r="D43" t="s">
-        <v>2</v>
+        <v>68</v>
+      </c>
+      <c r="D43">
+        <v>264.14999999999998</v>
       </c>
       <c r="E43" t="s">
         <v>2</v>
       </c>
       <c r="F43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G43" t="s">
         <v>2</v>
@@ -2200,48 +2266,433 @@
       <c r="I43">
         <v>0</v>
       </c>
-      <c r="J43">
-        <v>-395</v>
+      <c r="J43" t="s">
+        <v>2</v>
       </c>
       <c r="K43" t="s">
         <v>2</v>
       </c>
       <c r="L43">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>55</v>
+      </c>
+      <c r="C44" t="s">
+        <v>69</v>
+      </c>
+      <c r="D44">
+        <v>377.15</v>
+      </c>
+      <c r="E44" t="s">
+        <v>2</v>
+      </c>
+      <c r="F44">
+        <v>1</v>
+      </c>
+      <c r="G44">
+        <v>15.8992</v>
+      </c>
+      <c r="H44" t="s">
+        <v>2</v>
+      </c>
+      <c r="I44">
+        <v>1</v>
+      </c>
+      <c r="J44" t="s">
+        <v>2</v>
+      </c>
+      <c r="K44" t="s">
+        <v>2</v>
+      </c>
+      <c r="L44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>56</v>
+      </c>
+      <c r="C45" t="s">
+        <v>70</v>
+      </c>
+      <c r="D45" t="s">
+        <v>2</v>
+      </c>
+      <c r="E45" t="s">
+        <v>2</v>
+      </c>
+      <c r="F45">
+        <v>0</v>
+      </c>
+      <c r="G45" t="s">
+        <v>2</v>
+      </c>
+      <c r="H45" t="s">
+        <v>2</v>
+      </c>
+      <c r="I45">
+        <v>0</v>
+      </c>
+      <c r="J45">
+        <v>-256.83333333333331</v>
+      </c>
+      <c r="K45">
+        <v>9.6738479072876338</v>
+      </c>
+      <c r="L45">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>19</v>
+      </c>
+      <c r="C46" t="s">
+        <v>20</v>
+      </c>
+      <c r="D46">
+        <v>653.01</v>
+      </c>
+      <c r="E46">
+        <v>56.766532393656014</v>
+      </c>
+      <c r="F46">
+        <v>2</v>
+      </c>
+      <c r="G46">
+        <v>20.49</v>
+      </c>
+      <c r="H46" t="s">
+        <v>2</v>
+      </c>
+      <c r="I46">
+        <v>1</v>
+      </c>
+      <c r="J46">
+        <v>-274.8</v>
+      </c>
+      <c r="K46">
+        <v>2.4331050121192805</v>
+      </c>
+      <c r="L46">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>57</v>
+      </c>
+      <c r="C47" t="s">
+        <v>71</v>
+      </c>
+      <c r="D47" t="s">
+        <v>2</v>
+      </c>
+      <c r="E47" t="s">
+        <v>2</v>
+      </c>
+      <c r="F47">
+        <v>0</v>
+      </c>
+      <c r="G47" t="s">
+        <v>2</v>
+      </c>
+      <c r="H47" t="s">
+        <v>2</v>
+      </c>
+      <c r="I47">
+        <v>0</v>
+      </c>
+      <c r="J47">
+        <v>-199.13333333333333</v>
+      </c>
+      <c r="K47">
+        <v>7.9122268251948746</v>
+      </c>
+      <c r="L47">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>7</v>
+      </c>
+      <c r="C48" t="s">
+        <v>8</v>
+      </c>
+      <c r="D48">
+        <v>683</v>
+      </c>
+      <c r="E48" t="s">
+        <v>2</v>
+      </c>
+      <c r="F48">
+        <v>1</v>
+      </c>
+      <c r="G48">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="H48" t="s">
+        <v>2</v>
+      </c>
+      <c r="I48">
+        <v>1</v>
+      </c>
+      <c r="J48">
+        <v>-330.4</v>
+      </c>
+      <c r="K48">
+        <v>1.4071247279470325</v>
+      </c>
+      <c r="L48">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" t="s">
+        <v>72</v>
+      </c>
+      <c r="D49">
+        <v>376.15</v>
+      </c>
+      <c r="E49" t="s">
+        <v>2</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49">
+        <v>41.421600000000005</v>
+      </c>
+      <c r="H49" t="s">
+        <v>2</v>
+      </c>
+      <c r="I49">
+        <v>1</v>
+      </c>
+      <c r="J49" t="s">
+        <v>2</v>
+      </c>
+      <c r="K49" t="s">
+        <v>2</v>
+      </c>
+      <c r="L49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>59</v>
+      </c>
+      <c r="C50" t="s">
+        <v>73</v>
+      </c>
+      <c r="D50">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="E50" t="s">
+        <v>2</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50">
+        <v>1.29704</v>
+      </c>
+      <c r="H50" t="s">
+        <v>2</v>
+      </c>
+      <c r="I50">
+        <v>1</v>
+      </c>
+      <c r="J50" t="s">
+        <v>2</v>
+      </c>
+      <c r="K50" t="s">
+        <v>2</v>
+      </c>
+      <c r="L50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>60</v>
+      </c>
+      <c r="C51" t="s">
+        <v>74</v>
+      </c>
+      <c r="D51">
+        <v>412.15</v>
+      </c>
+      <c r="E51" t="s">
+        <v>2</v>
+      </c>
+      <c r="F51">
+        <v>1</v>
+      </c>
+      <c r="G51">
+        <v>39.329600000000006</v>
+      </c>
+      <c r="H51" t="s">
+        <v>2</v>
+      </c>
+      <c r="I51">
+        <v>1</v>
+      </c>
+      <c r="J51" t="s">
+        <v>2</v>
+      </c>
+      <c r="K51" t="s">
+        <v>2</v>
+      </c>
+      <c r="L51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>61</v>
+      </c>
+      <c r="C52" t="s">
+        <v>75</v>
+      </c>
+      <c r="D52" t="s">
+        <v>2</v>
+      </c>
+      <c r="E52" t="s">
+        <v>2</v>
+      </c>
+      <c r="F52">
+        <v>0</v>
+      </c>
+      <c r="G52" t="s">
+        <v>2</v>
+      </c>
+      <c r="H52" t="s">
+        <v>2</v>
+      </c>
+      <c r="I52">
+        <v>0</v>
+      </c>
+      <c r="J52">
+        <v>-442</v>
+      </c>
+      <c r="K52" t="s">
+        <v>2</v>
+      </c>
+      <c r="L52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>21</v>
+      </c>
+      <c r="C53" t="s">
+        <v>22</v>
+      </c>
+      <c r="D53">
+        <v>459.61</v>
+      </c>
+      <c r="E53">
+        <v>61.461721420734726</v>
+      </c>
+      <c r="F53">
+        <v>2</v>
+      </c>
+      <c r="G53">
+        <v>66.58</v>
+      </c>
+      <c r="H53" t="s">
+        <v>2</v>
+      </c>
+      <c r="I53">
+        <v>1</v>
+      </c>
+      <c r="J53">
+        <v>-487.5</v>
+      </c>
+      <c r="K53">
+        <v>17.677669529663689</v>
+      </c>
+      <c r="L53">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>62</v>
+      </c>
+      <c r="C54" t="s">
+        <v>76</v>
+      </c>
+      <c r="D54" t="s">
+        <v>2</v>
+      </c>
+      <c r="E54" t="s">
+        <v>2</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+      <c r="G54" t="s">
+        <v>2</v>
+      </c>
+      <c r="H54" t="s">
+        <v>2</v>
+      </c>
+      <c r="I54">
+        <v>0</v>
+      </c>
+      <c r="J54">
+        <v>-395</v>
+      </c>
+      <c r="K54" t="s">
+        <v>2</v>
+      </c>
+      <c r="L54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>41</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C55" t="s">
         <v>42</v>
       </c>
-      <c r="D44">
+      <c r="D55">
         <v>153.26</v>
       </c>
-      <c r="E44">
+      <c r="E55">
         <v>3.6390932936653244</v>
       </c>
-      <c r="F44">
+      <c r="F55">
         <v>5</v>
       </c>
-      <c r="G44">
+      <c r="G55">
         <v>6.5419999999999998</v>
       </c>
-      <c r="H44">
+      <c r="H55">
         <v>2.8284271247458787E-3</v>
       </c>
-      <c r="I44">
-        <v>2</v>
-      </c>
-      <c r="J44">
+      <c r="I55">
+        <v>2</v>
+      </c>
+      <c r="J55">
         <v>-27.2</v>
       </c>
-      <c r="K44">
+      <c r="K55">
         <v>4.9497474683058327</v>
       </c>
-      <c r="L44">
+      <c r="L55">
         <v>2</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Flattened out the target into 1D with a task index to avoid issues with missing data.
</commit_message>
<xml_diff>
--- a/MTGPR_train.xlsx
+++ b/MTGPR_train.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03D0664E-13FA-4515-B364-52EF6EEF08F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C04DD60-2BF0-4223-ADB3-187E149DCFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
@@ -38,8 +38,43 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Alexander Glotov</author>
+  </authors>
+  <commentList>
+    <comment ref="P56" authorId="0" shapeId="0" xr:uid="{C2877B65-457A-4757-ADC7-454520251F31}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Alexander Glotov:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+Source(s):
+1)https://matweb.com/search/datasheet.aspx?MatGUID=3118b2052ace4835a6d73687613def66&amp;ckck=1</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="115">
   <si>
     <t>tetrabutylammonium bromide</t>
   </si>
@@ -170,6 +205,12 @@
     <t>CN(C)C</t>
   </si>
   <si>
+    <t>Lithium Borohydride</t>
+  </si>
+  <si>
+    <t>[BH4-].[Li+]</t>
+  </si>
+  <si>
     <t>acetonitrile</t>
   </si>
   <si>
@@ -341,9 +382,6 @@
     <t>dihydrogen</t>
   </si>
   <si>
-    <t>[HH]</t>
-  </si>
-  <si>
     <t>dinitrogen</t>
   </si>
   <si>
@@ -378,6 +416,9 @@
   </si>
   <si>
     <t>[S]</t>
+  </si>
+  <si>
+    <t>[H][H]</t>
   </si>
 </sst>
 </file>
@@ -387,7 +428,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -399,6 +440,19 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -784,8 +838,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
-  <dimension ref="A1:L55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
+  <dimension ref="A1:P56"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -808,10 +862,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D2">
         <v>228</v>
@@ -878,10 +932,10 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D4">
         <v>263</v>
@@ -913,10 +967,10 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D5">
         <v>2349.15</v>
@@ -948,10 +1002,10 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D6">
         <v>160.91</v>
@@ -983,10 +1037,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C7" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D7">
         <v>1115.1500000000001</v>
@@ -1018,10 +1072,10 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D8" t="s">
         <v>2</v>
@@ -1053,10 +1107,10 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D9">
         <v>245.31</v>
@@ -1088,10 +1142,10 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D10">
         <v>171.64999999999998</v>
@@ -1123,10 +1177,10 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C11" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="D11">
         <v>14.009999999999991</v>
@@ -1193,10 +1247,10 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C13" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D13">
         <v>215.97499999999999</v>
@@ -1228,10 +1282,10 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D14">
         <v>63.049999999999983</v>
@@ -1263,10 +1317,10 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C15" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D15">
         <v>263.84999999999997</v>
@@ -1298,10 +1352,10 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D16">
         <v>327.95</v>
@@ -1368,10 +1422,10 @@
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C18" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D18">
         <v>155</v>
@@ -1438,10 +1492,10 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C20" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D20">
         <v>162.17500000000001</v>
@@ -1473,10 +1527,10 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D21">
         <v>274.93333333333334</v>
@@ -1508,10 +1562,10 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C22" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D22">
         <v>453.68999999999994</v>
@@ -1718,10 +1772,10 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D28">
         <v>220.79500000000002</v>
@@ -1753,10 +1807,10 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C29" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D29">
         <v>336.53</v>
@@ -1788,10 +1842,10 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C30" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D30">
         <v>180</v>
@@ -1858,10 +1912,10 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C32" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D32">
         <v>370.87</v>
@@ -1893,10 +1947,10 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D33">
         <v>368.45</v>
@@ -1963,10 +2017,10 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C35" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D35">
         <v>314.14999999999998</v>
@@ -2068,10 +2122,10 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C38" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="D38">
         <v>502.2</v>
@@ -2173,10 +2227,10 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C41" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D41" t="s">
         <v>2</v>
@@ -2208,10 +2262,10 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="C42" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D42" t="s">
         <v>2</v>
@@ -2243,10 +2297,10 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C43" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D43">
         <v>264.14999999999998</v>
@@ -2278,10 +2332,10 @@
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C44" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D44">
         <v>377.15</v>
@@ -2313,10 +2367,10 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C45" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D45" t="s">
         <v>2</v>
@@ -2383,10 +2437,10 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C47" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D47" t="s">
         <v>2</v>
@@ -2451,12 +2505,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C49" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="D49">
         <v>376.15</v>
@@ -2486,12 +2540,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C50" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D50">
         <v>295.14999999999998</v>
@@ -2521,12 +2575,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C51" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D51">
         <v>412.15</v>
@@ -2556,12 +2610,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C52" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D52" t="s">
         <v>2</v>
@@ -2591,7 +2645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>21</v>
       </c>
@@ -2626,12 +2680,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C54" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D54" t="s">
         <v>2</v>
@@ -2661,7 +2715,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>41</v>
       </c>
@@ -2694,6 +2748,33 @@
       </c>
       <c r="L55">
         <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C56" t="s">
+        <v>44</v>
+      </c>
+      <c r="D56">
+        <f>273.15+286</f>
+        <v>559.15</v>
+      </c>
+      <c r="G56">
+        <f>O56/1000</f>
+        <v>7.14</v>
+      </c>
+      <c r="J56">
+        <f>P56/1000</f>
+        <v>-190.8</v>
+      </c>
+      <c r="O56">
+        <f>AVERAGE(7.56,6.72)*1000</f>
+        <v>7140</v>
+      </c>
+      <c r="P56">
+        <v>-190800</v>
       </c>
     </row>
   </sheetData>
@@ -2706,5 +2787,6 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Adjusted the priors covariance and the method for tier 2 selection.
</commit_message>
<xml_diff>
--- a/MTGPR_train.xlsx
+++ b/MTGPR_train.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\aglotov\Eutectics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C04DD60-2BF0-4223-ADB3-187E149DCFBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3425D11B-D1F1-4C16-8B10-9DE02DF3815D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{535DD4A0-2912-47A9-820B-218FC7178EC0}"/>
   </bookViews>
@@ -38,43 +38,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Alexander Glotov</author>
-  </authors>
-  <commentList>
-    <comment ref="P56" authorId="0" shapeId="0" xr:uid="{C2877B65-457A-4757-ADC7-454520251F31}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Alexander Glotov:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-Source(s):
-1)https://matweb.com/search/datasheet.aspx?MatGUID=3118b2052ace4835a6d73687613def66&amp;ckck=1</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="117">
   <si>
     <t>tetrabutylammonium bromide</t>
   </si>
@@ -205,9 +170,6 @@
     <t>CN(C)C</t>
   </si>
   <si>
-    <t>Lithium Borohydride</t>
-  </si>
-  <si>
     <t>[BH4-].[Li+]</t>
   </si>
   <si>
@@ -419,6 +381,15 @@
   </si>
   <si>
     <t>[H][H]</t>
+  </si>
+  <si>
+    <t>[BH4-].[K+]</t>
+  </si>
+  <si>
+    <t>lithium borohydride</t>
+  </si>
+  <si>
+    <t>potassium borohydride</t>
   </si>
 </sst>
 </file>
@@ -428,7 +399,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -440,19 +411,6 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -838,8 +796,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
-  <dimension ref="A1:P56"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB4AABDE-AFF5-4072-A990-39ABD46EABEB}">
+  <dimension ref="A1:L57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="36.42578125" bestFit="1" customWidth="1"/>
@@ -862,10 +820,10 @@
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D2">
         <v>228</v>
@@ -932,10 +890,10 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" t="s">
         <v>79</v>
-      </c>
-      <c r="C4" t="s">
-        <v>80</v>
       </c>
       <c r="D4">
         <v>263</v>
@@ -967,19 +925,19 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" t="s">
         <v>93</v>
       </c>
-      <c r="C5" t="s">
-        <v>94</v>
-      </c>
       <c r="D5">
-        <v>2349.15</v>
-      </c>
-      <c r="E5" t="s">
-        <v>2</v>
+        <v>2348.8166666666671</v>
+      </c>
+      <c r="E5">
+        <v>0.57735026918962573</v>
       </c>
       <c r="F5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G5">
         <v>50.133333333333333</v>
@@ -1001,11 +959,11 @@
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C6" t="s">
         <v>81</v>
-      </c>
-      <c r="C6" t="s">
-        <v>82</v>
       </c>
       <c r="D6">
         <v>160.91</v>
@@ -1036,20 +994,20 @@
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" t="s">
         <v>95</v>
-      </c>
-      <c r="C7" t="s">
-        <v>96</v>
       </c>
       <c r="D7">
         <v>1115.1500000000001</v>
       </c>
-      <c r="E7" t="s">
-        <v>2</v>
+      <c r="E7">
+        <v>0</v>
       </c>
       <c r="F7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G7">
         <v>8.5399999999999991</v>
@@ -1071,11 +1029,11 @@
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C8" t="s">
         <v>97</v>
-      </c>
-      <c r="C8" t="s">
-        <v>98</v>
       </c>
       <c r="D8" t="s">
         <v>2</v>
@@ -1106,11 +1064,11 @@
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C9" t="s">
         <v>83</v>
-      </c>
-      <c r="C9" t="s">
-        <v>84</v>
       </c>
       <c r="D9">
         <v>245.31</v>
@@ -1142,19 +1100,19 @@
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" t="s">
         <v>99</v>
-      </c>
-      <c r="C10" t="s">
-        <v>100</v>
       </c>
       <c r="D10">
         <v>171.64999999999998</v>
       </c>
-      <c r="E10" t="s">
-        <v>2</v>
+      <c r="E10">
+        <v>0</v>
       </c>
       <c r="F10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G10">
         <v>6.4030000000000005</v>
@@ -1177,19 +1135,19 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D11">
-        <v>14.009999999999991</v>
-      </c>
-      <c r="E11" t="s">
-        <v>2</v>
+        <v>13.9333333333333</v>
+      </c>
+      <c r="E11">
+        <v>0.11590225767143621</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G11">
         <v>0.11849999999999999</v>
@@ -1247,10 +1205,10 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="C13" t="s">
         <v>85</v>
-      </c>
-      <c r="C13" t="s">
-        <v>86</v>
       </c>
       <c r="D13">
         <v>215.97499999999999</v>
@@ -1282,19 +1240,19 @@
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" t="s">
         <v>102</v>
       </c>
-      <c r="C14" t="s">
-        <v>103</v>
-      </c>
       <c r="D14">
-        <v>63.049999999999983</v>
-      </c>
-      <c r="E14" t="s">
-        <v>2</v>
+        <v>63.113333333333316</v>
+      </c>
+      <c r="E14">
+        <v>5.5075705472859955E-2</v>
       </c>
       <c r="F14">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G14">
         <v>0.71499999999999997</v>
@@ -1317,10 +1275,10 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C15" t="s">
         <v>87</v>
-      </c>
-      <c r="C15" t="s">
-        <v>88</v>
       </c>
       <c r="D15">
         <v>263.84999999999997</v>
@@ -1352,10 +1310,10 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16" t="s">
         <v>104</v>
-      </c>
-      <c r="C16" t="s">
-        <v>105</v>
       </c>
       <c r="D16">
         <v>327.95</v>
@@ -1386,7 +1344,7 @@
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="A17" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C17" t="s">
@@ -1421,11 +1379,11 @@
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="A18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" t="s">
         <v>46</v>
-      </c>
-      <c r="C18" t="s">
-        <v>47</v>
       </c>
       <c r="D18">
         <v>155</v>
@@ -1456,7 +1414,7 @@
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C19" t="s">
@@ -1491,11 +1449,11 @@
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="A20" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C20" t="s">
         <v>48</v>
-      </c>
-      <c r="C20" t="s">
-        <v>49</v>
       </c>
       <c r="D20">
         <v>162.17500000000001</v>
@@ -1527,10 +1485,10 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C21" t="s">
         <v>89</v>
-      </c>
-      <c r="C21" t="s">
-        <v>90</v>
       </c>
       <c r="D21">
         <v>274.93333333333334</v>
@@ -1550,10 +1508,10 @@
       <c r="I21">
         <v>0</v>
       </c>
-      <c r="J21">
+      <c r="J21" s="2">
         <v>50.63</v>
       </c>
-      <c r="K21" t="s">
+      <c r="K21" s="2" t="s">
         <v>2</v>
       </c>
       <c r="L21">
@@ -1562,19 +1520,19 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C22" t="s">
         <v>106</v>
       </c>
-      <c r="C22" t="s">
-        <v>107</v>
-      </c>
       <c r="D22">
-        <v>453.68999999999994</v>
-      </c>
-      <c r="E22" t="s">
-        <v>2</v>
+        <v>453.67666666666656</v>
+      </c>
+      <c r="E22">
+        <v>2.3094010767564028E-2</v>
       </c>
       <c r="F22">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G22">
         <v>3</v>
@@ -1585,10 +1543,10 @@
       <c r="I22">
         <v>3</v>
       </c>
-      <c r="J22">
-        <v>0</v>
-      </c>
-      <c r="K22" t="s">
+      <c r="J22" s="2">
+        <v>0</v>
+      </c>
+      <c r="K22" s="2" t="s">
         <v>2</v>
       </c>
       <c r="L22">
@@ -1597,22 +1555,22 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>29</v>
+        <v>115</v>
       </c>
       <c r="C23" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="D23">
-        <v>89.72</v>
-      </c>
-      <c r="E23">
-        <v>2.2642879675518288</v>
+        <v>559.15</v>
+      </c>
+      <c r="E23" t="s">
+        <v>2</v>
       </c>
       <c r="F23">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G23">
-        <v>0.93920000000000003</v>
+        <v>7.14</v>
       </c>
       <c r="H23" t="s">
         <v>2</v>
@@ -1620,80 +1578,80 @@
       <c r="I23">
         <v>1</v>
       </c>
-      <c r="J23">
-        <v>-74.444000000000003</v>
-      </c>
-      <c r="K23">
-        <v>0.60492148250826439</v>
+      <c r="J23" s="2">
+        <v>-190.8</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L23">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24">
+        <v>89.72</v>
+      </c>
+      <c r="E24">
+        <v>2.2642879675518288</v>
+      </c>
+      <c r="F24">
+        <v>5</v>
+      </c>
+      <c r="G24">
+        <v>0.93920000000000003</v>
+      </c>
+      <c r="H24" t="s">
+        <v>2</v>
+      </c>
+      <c r="I24">
+        <v>1</v>
+      </c>
+      <c r="J24" s="2">
+        <v>-74.444000000000003</v>
+      </c>
+      <c r="K24" s="2">
+        <v>0.60492148250826439</v>
+      </c>
+      <c r="L24">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>31</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C25" t="s">
         <v>32</v>
       </c>
-      <c r="D24">
+      <c r="D25">
         <v>179.5</v>
       </c>
-      <c r="E24" t="s">
-        <v>2</v>
-      </c>
-      <c r="F24">
-        <v>1</v>
-      </c>
-      <c r="G24">
+      <c r="E25" t="s">
+        <v>2</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25">
         <v>5.98</v>
       </c>
-      <c r="H24" t="s">
-        <v>2</v>
-      </c>
-      <c r="I24">
-        <v>1</v>
-      </c>
-      <c r="J24">
+      <c r="H25" t="s">
+        <v>2</v>
+      </c>
+      <c r="I25">
+        <v>1</v>
+      </c>
+      <c r="J25" s="2">
         <v>-60.6</v>
       </c>
-      <c r="K24" t="s">
-        <v>2</v>
-      </c>
-      <c r="L24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C25" t="s">
-        <v>34</v>
-      </c>
-      <c r="D25">
-        <v>178.01666666666665</v>
-      </c>
-      <c r="E25">
-        <v>3.4822167269331912</v>
-      </c>
-      <c r="F25">
-        <v>3</v>
-      </c>
-      <c r="G25">
-        <v>6.4254999999999995</v>
-      </c>
-      <c r="H25">
-        <v>7.778174593052108E-3</v>
-      </c>
-      <c r="I25">
-        <v>2</v>
-      </c>
-      <c r="J25">
-        <v>-102.4</v>
-      </c>
-      <c r="K25" t="s">
+      <c r="K25" s="2" t="s">
         <v>2</v>
       </c>
       <c r="L25">
@@ -1702,69 +1660,69 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C26" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D26">
-        <v>207.39999999999998</v>
+        <v>178.01666666666665</v>
       </c>
       <c r="E26">
-        <v>0.98994949366117058</v>
+        <v>3.4822167269331912</v>
       </c>
       <c r="F26">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G26">
-        <v>9.1199999999999992</v>
-      </c>
-      <c r="H26" t="s">
-        <v>2</v>
+        <v>6.4254999999999995</v>
+      </c>
+      <c r="H26">
+        <v>7.778174593052108E-3</v>
       </c>
       <c r="I26">
-        <v>1</v>
-      </c>
-      <c r="J26">
-        <v>-12.8</v>
-      </c>
-      <c r="K26">
-        <v>1.1313708498984758</v>
+        <v>2</v>
+      </c>
+      <c r="J26" s="2">
+        <v>-102.4</v>
+      </c>
+      <c r="K26" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L26">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C27" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D27">
-        <v>179.93333333333331</v>
+        <v>207.39999999999998</v>
       </c>
       <c r="E27">
-        <v>0.20207259421638213</v>
+        <v>0.98994949366117058</v>
       </c>
       <c r="F27">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G27">
-        <v>6.1319999999999997</v>
-      </c>
-      <c r="H27">
-        <v>2.8284271247465066E-3</v>
+        <v>9.1199999999999992</v>
+      </c>
+      <c r="H27" t="s">
+        <v>2</v>
       </c>
       <c r="I27">
-        <v>2</v>
-      </c>
-      <c r="J27">
-        <v>-17.850000000000001</v>
-      </c>
-      <c r="K27">
-        <v>7.9903066274079748</v>
+        <v>1</v>
+      </c>
+      <c r="J27" s="2">
+        <v>-12.8</v>
+      </c>
+      <c r="K27" s="2">
+        <v>1.1313708498984758</v>
       </c>
       <c r="L27">
         <v>2</v>
@@ -1772,68 +1730,68 @@
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>91</v>
+        <v>37</v>
       </c>
       <c r="C28" t="s">
-        <v>92</v>
+        <v>38</v>
       </c>
       <c r="D28">
-        <v>220.79500000000002</v>
+        <v>179.93333333333331</v>
       </c>
       <c r="E28">
-        <v>7.0710678118791415E-3</v>
+        <v>0.20207259421638213</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G28">
-        <v>10.419</v>
+        <v>6.1319999999999997</v>
       </c>
       <c r="H28">
-        <v>1.4142135623735675E-3</v>
+        <v>2.8284271247465066E-3</v>
       </c>
       <c r="I28">
         <v>2</v>
       </c>
-      <c r="J28">
-        <v>54.14</v>
-      </c>
-      <c r="K28" t="s">
-        <v>2</v>
+      <c r="J28" s="2">
+        <v>-17.850000000000001</v>
+      </c>
+      <c r="K28" s="2">
+        <v>7.9903066274079748</v>
       </c>
       <c r="L28">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="C29" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="D29">
-        <v>336.53</v>
-      </c>
-      <c r="E29" t="s">
-        <v>2</v>
+        <v>220.79500000000002</v>
+      </c>
+      <c r="E29">
+        <v>7.0710678118791415E-3</v>
       </c>
       <c r="F29">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29">
-        <v>2.327</v>
+        <v>10.419</v>
       </c>
       <c r="H29">
-        <v>5.1961524227065728E-3</v>
+        <v>1.4142135623735675E-3</v>
       </c>
       <c r="I29">
-        <v>3</v>
-      </c>
-      <c r="J29">
-        <v>0</v>
-      </c>
-      <c r="K29" t="s">
+        <v>2</v>
+      </c>
+      <c r="J29" s="2">
+        <v>54.14</v>
+      </c>
+      <c r="K29" s="2" t="s">
         <v>2</v>
       </c>
       <c r="L29">
@@ -1842,33 +1800,33 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>50</v>
+        <v>107</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>108</v>
       </c>
       <c r="D30">
-        <v>180</v>
-      </c>
-      <c r="E30" t="s">
-        <v>2</v>
+        <v>336.57</v>
+      </c>
+      <c r="E30">
+        <v>6.9282032302757715E-2</v>
       </c>
       <c r="F30">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G30">
-        <v>5.03</v>
-      </c>
-      <c r="H30" t="s">
-        <v>2</v>
+        <v>2.327</v>
+      </c>
+      <c r="H30">
+        <v>5.1961524227065728E-3</v>
       </c>
       <c r="I30">
-        <v>1</v>
-      </c>
-      <c r="J30">
-        <v>15.5</v>
-      </c>
-      <c r="K30" t="s">
+        <v>3</v>
+      </c>
+      <c r="J30" s="2">
+        <v>0</v>
+      </c>
+      <c r="K30" s="2" t="s">
         <v>2</v>
       </c>
       <c r="L30">
@@ -1877,13 +1835,13 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>116</v>
       </c>
       <c r="C31" t="s">
-        <v>40</v>
+        <v>114</v>
       </c>
       <c r="D31">
-        <v>190.15</v>
+        <v>878.15</v>
       </c>
       <c r="E31" t="s">
         <v>2</v>
@@ -1892,33 +1850,33 @@
         <v>1</v>
       </c>
       <c r="G31">
-        <v>10.856400000000001</v>
-      </c>
-      <c r="H31">
-        <v>0.20040928122220297</v>
+        <v>19.2</v>
+      </c>
+      <c r="H31" t="s">
+        <v>2</v>
       </c>
       <c r="I31">
-        <v>3</v>
-      </c>
-      <c r="J31">
-        <v>-119.75</v>
-      </c>
-      <c r="K31">
-        <v>25.809397513308983</v>
+        <v>1</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K31" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L31">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>110</v>
+        <v>49</v>
       </c>
       <c r="C32" t="s">
-        <v>111</v>
+        <v>65</v>
       </c>
       <c r="D32">
-        <v>370.87</v>
+        <v>180</v>
       </c>
       <c r="E32" t="s">
         <v>2</v>
@@ -1927,18 +1885,18 @@
         <v>1</v>
       </c>
       <c r="G32">
-        <v>2.6</v>
-      </c>
-      <c r="H32">
-        <v>0</v>
+        <v>5.03</v>
+      </c>
+      <c r="H32" t="s">
+        <v>2</v>
       </c>
       <c r="I32">
-        <v>3</v>
-      </c>
-      <c r="J32">
-        <v>0</v>
-      </c>
-      <c r="K32" t="s">
+        <v>1</v>
+      </c>
+      <c r="J32" s="2">
+        <v>15.5</v>
+      </c>
+      <c r="K32" s="2" t="s">
         <v>2</v>
       </c>
       <c r="L32">
@@ -1947,13 +1905,13 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>112</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s">
-        <v>113</v>
+        <v>40</v>
       </c>
       <c r="D33">
-        <v>368.45</v>
+        <v>190.15</v>
       </c>
       <c r="E33" t="s">
         <v>2</v>
@@ -1962,124 +1920,124 @@
         <v>1</v>
       </c>
       <c r="G33">
-        <v>1.7256666666666665</v>
+        <v>10.856400000000001</v>
       </c>
       <c r="H33">
-        <v>5.1316014394469037E-3</v>
+        <v>0.20040928122220297</v>
       </c>
       <c r="I33">
         <v>3</v>
       </c>
-      <c r="J33">
-        <v>0</v>
-      </c>
-      <c r="K33" t="s">
-        <v>2</v>
+      <c r="J33" s="2">
+        <v>-119.75</v>
+      </c>
+      <c r="K33" s="2">
+        <v>25.809397513308983</v>
       </c>
       <c r="L33">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>0</v>
+        <v>109</v>
       </c>
       <c r="C34" t="s">
-        <v>1</v>
+        <v>110</v>
       </c>
       <c r="D34">
-        <v>395.07499999999999</v>
+        <v>370.92799999999994</v>
       </c>
       <c r="E34">
-        <v>0.10606601717796604</v>
+        <v>5.1884487084270715E-2</v>
       </c>
       <c r="F34">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G34">
-        <v>15.8154</v>
+        <v>2.6</v>
       </c>
       <c r="H34">
-        <v>0.47319585797003511</v>
+        <v>0</v>
       </c>
       <c r="I34">
-        <v>2</v>
-      </c>
-      <c r="J34">
-        <v>-477.65</v>
-      </c>
-      <c r="K34">
-        <v>88.600479682674319</v>
+        <v>3</v>
+      </c>
+      <c r="J34" s="2">
+        <v>0</v>
+      </c>
+      <c r="K34" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L34">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>51</v>
+        <v>111</v>
       </c>
       <c r="C35" t="s">
-        <v>52</v>
+        <v>112</v>
       </c>
       <c r="D35">
-        <v>314.14999999999998</v>
-      </c>
-      <c r="E35" t="s">
-        <v>2</v>
+        <v>378.92</v>
+      </c>
+      <c r="E35">
+        <v>9.9948836911691821</v>
       </c>
       <c r="F35">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G35">
-        <v>20.501600000000003</v>
-      </c>
-      <c r="H35" t="s">
-        <v>2</v>
+        <v>1.7256666666666665</v>
+      </c>
+      <c r="H35">
+        <v>5.1316014394469037E-3</v>
       </c>
       <c r="I35">
-        <v>1</v>
-      </c>
-      <c r="J35">
-        <v>-549.4</v>
-      </c>
-      <c r="K35">
-        <v>21.778888860545631</v>
+        <v>3</v>
+      </c>
+      <c r="J35" s="2">
+        <v>0</v>
+      </c>
+      <c r="K35" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L35">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C36" t="s">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D36">
-        <v>419.15</v>
-      </c>
-      <c r="E36" t="s">
-        <v>2</v>
+        <v>395.07499999999999</v>
+      </c>
+      <c r="E36">
+        <v>0.10606601717796604</v>
       </c>
       <c r="F36">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G36">
-        <v>9.6231999999999989</v>
-      </c>
-      <c r="H36" t="s">
-        <v>2</v>
+        <v>15.8154</v>
+      </c>
+      <c r="H36">
+        <v>0.47319585797003511</v>
       </c>
       <c r="I36">
-        <v>1</v>
-      </c>
-      <c r="J36">
-        <v>-479.3</v>
-      </c>
-      <c r="K36">
-        <v>27.294321753800752</v>
+        <v>2</v>
+      </c>
+      <c r="J36" s="2">
+        <v>-477.65</v>
+      </c>
+      <c r="K36" s="2">
+        <v>88.600479682674319</v>
       </c>
       <c r="L36">
         <v>2</v>
@@ -2087,48 +2045,48 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="C37" t="s">
-        <v>6</v>
+        <v>51</v>
       </c>
       <c r="D37">
-        <v>389.9666666666667</v>
-      </c>
-      <c r="E37">
-        <v>1.9857828011475314</v>
+        <v>314.14999999999998</v>
+      </c>
+      <c r="E37" t="s">
+        <v>2</v>
       </c>
       <c r="F37">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G37">
-        <v>14.95</v>
-      </c>
-      <c r="H37">
-        <v>0.91923881554251108</v>
+        <v>20.501600000000003</v>
+      </c>
+      <c r="H37" t="s">
+        <v>2</v>
       </c>
       <c r="I37">
-        <v>2</v>
-      </c>
-      <c r="J37">
-        <v>-600.20000000000005</v>
-      </c>
-      <c r="K37" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="J37" s="2">
+        <v>-549.4</v>
+      </c>
+      <c r="K37" s="2">
+        <v>21.778888860545631</v>
       </c>
       <c r="L37">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>53</v>
+        <v>3</v>
       </c>
       <c r="C38" t="s">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="D38">
-        <v>502.2</v>
+        <v>419.15</v>
       </c>
       <c r="E38" t="s">
         <v>2</v>
@@ -2136,69 +2094,69 @@
       <c r="F38">
         <v>1</v>
       </c>
-      <c r="G38" t="s">
-        <v>2</v>
+      <c r="G38">
+        <v>9.6231999999999989</v>
       </c>
       <c r="H38" t="s">
         <v>2</v>
       </c>
       <c r="I38">
-        <v>0</v>
-      </c>
-      <c r="J38" t="s">
-        <v>2</v>
-      </c>
-      <c r="K38" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="J38" s="2">
+        <v>-479.3</v>
+      </c>
+      <c r="K38" s="2">
+        <v>27.294321753800752</v>
       </c>
       <c r="L38">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="C39" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="D39">
-        <v>447</v>
-      </c>
-      <c r="E39" t="s">
-        <v>2</v>
+        <v>389.9666666666667</v>
+      </c>
+      <c r="E39">
+        <v>1.9857828011475314</v>
       </c>
       <c r="F39">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G39">
-        <v>20.3</v>
-      </c>
-      <c r="H39" t="s">
-        <v>2</v>
+        <v>14.95</v>
+      </c>
+      <c r="H39">
+        <v>0.91923881554251108</v>
       </c>
       <c r="I39">
-        <v>1</v>
-      </c>
-      <c r="J39">
-        <v>-363.45</v>
-      </c>
-      <c r="K39">
-        <v>15.700212312789498</v>
+        <v>2</v>
+      </c>
+      <c r="J39" s="2">
+        <v>-600.20000000000005</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L39">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="C40" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="D40">
-        <v>526.78</v>
+        <v>502.2</v>
       </c>
       <c r="E40" t="s">
         <v>2</v>
@@ -2206,55 +2164,55 @@
       <c r="F40">
         <v>1</v>
       </c>
-      <c r="G40">
-        <v>51.24</v>
+      <c r="G40" t="s">
+        <v>2</v>
       </c>
       <c r="H40" t="s">
         <v>2</v>
       </c>
       <c r="I40">
-        <v>1</v>
-      </c>
-      <c r="J40">
-        <v>-396.29999999999995</v>
-      </c>
-      <c r="K40">
-        <v>18.966988866624746</v>
+        <v>0</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L40">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="C41" t="s">
-        <v>68</v>
-      </c>
-      <c r="D41" t="s">
-        <v>2</v>
+        <v>16</v>
+      </c>
+      <c r="D41">
+        <v>447</v>
       </c>
       <c r="E41" t="s">
         <v>2</v>
       </c>
       <c r="F41">
-        <v>0</v>
-      </c>
-      <c r="G41" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G41">
+        <v>20.3</v>
       </c>
       <c r="H41" t="s">
         <v>2</v>
       </c>
       <c r="I41">
-        <v>0</v>
-      </c>
-      <c r="J41">
-        <v>-316.17500000000001</v>
-      </c>
-      <c r="K41">
-        <v>12.790198069876276</v>
+        <v>1</v>
+      </c>
+      <c r="J41" s="2">
+        <v>-363.45</v>
+      </c>
+      <c r="K41" s="2">
+        <v>15.700212312789498</v>
       </c>
       <c r="L41">
         <v>4</v>
@@ -2262,54 +2220,54 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>55</v>
+        <v>17</v>
       </c>
       <c r="C42" t="s">
-        <v>69</v>
-      </c>
-      <c r="D42" t="s">
-        <v>2</v>
+        <v>18</v>
+      </c>
+      <c r="D42">
+        <v>526.78</v>
       </c>
       <c r="E42" t="s">
         <v>2</v>
       </c>
       <c r="F42">
-        <v>0</v>
-      </c>
-      <c r="G42" t="s">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G42">
+        <v>51.24</v>
       </c>
       <c r="H42" t="s">
         <v>2</v>
       </c>
       <c r="I42">
-        <v>0</v>
-      </c>
-      <c r="J42">
-        <v>-430.83333333333331</v>
-      </c>
-      <c r="K42">
-        <v>2.2546248764114472</v>
+        <v>1</v>
+      </c>
+      <c r="J42" s="2">
+        <v>-396.29999999999995</v>
+      </c>
+      <c r="K42" s="2">
+        <v>18.966988866624746</v>
       </c>
       <c r="L42">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C43" t="s">
-        <v>70</v>
-      </c>
-      <c r="D43">
-        <v>264.14999999999998</v>
+        <v>67</v>
+      </c>
+      <c r="D43" t="s">
+        <v>2</v>
       </c>
       <c r="E43" t="s">
         <v>2</v>
       </c>
       <c r="F43">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G43" t="s">
         <v>2</v>
@@ -2320,66 +2278,66 @@
       <c r="I43">
         <v>0</v>
       </c>
-      <c r="J43" t="s">
-        <v>2</v>
-      </c>
-      <c r="K43" t="s">
-        <v>2</v>
+      <c r="J43" s="2">
+        <v>-316.17500000000001</v>
+      </c>
+      <c r="K43" s="2">
+        <v>12.790198069876276</v>
       </c>
       <c r="L43">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C44" t="s">
-        <v>71</v>
-      </c>
-      <c r="D44">
-        <v>377.15</v>
+        <v>68</v>
+      </c>
+      <c r="D44" t="s">
+        <v>2</v>
       </c>
       <c r="E44" t="s">
         <v>2</v>
       </c>
       <c r="F44">
-        <v>1</v>
-      </c>
-      <c r="G44">
-        <v>15.8992</v>
+        <v>0</v>
+      </c>
+      <c r="G44" t="s">
+        <v>2</v>
       </c>
       <c r="H44" t="s">
         <v>2</v>
       </c>
       <c r="I44">
-        <v>1</v>
-      </c>
-      <c r="J44" t="s">
-        <v>2</v>
-      </c>
-      <c r="K44" t="s">
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="J44" s="2">
+        <v>-430.83333333333331</v>
+      </c>
+      <c r="K44" s="2">
+        <v>2.2546248764114472</v>
       </c>
       <c r="L44">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C45" t="s">
-        <v>72</v>
-      </c>
-      <c r="D45" t="s">
-        <v>2</v>
+        <v>69</v>
+      </c>
+      <c r="D45">
+        <v>264.14999999999998</v>
       </c>
       <c r="E45" t="s">
         <v>2</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G45" t="s">
         <v>2</v>
@@ -2390,34 +2348,34 @@
       <c r="I45">
         <v>0</v>
       </c>
-      <c r="J45">
-        <v>-256.83333333333331</v>
-      </c>
-      <c r="K45">
-        <v>9.6738479072876338</v>
+      <c r="J45" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K45" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L45">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="C46" t="s">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="D46">
-        <v>653.01</v>
-      </c>
-      <c r="E46">
-        <v>56.766532393656014</v>
+        <v>377.15</v>
+      </c>
+      <c r="E46" t="s">
+        <v>2</v>
       </c>
       <c r="F46">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G46">
-        <v>20.49</v>
+        <v>15.8992</v>
       </c>
       <c r="H46" t="s">
         <v>2</v>
@@ -2425,22 +2383,22 @@
       <c r="I46">
         <v>1</v>
       </c>
-      <c r="J46">
-        <v>-274.8</v>
-      </c>
-      <c r="K46">
-        <v>2.4331050121192805</v>
+      <c r="J46" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>2</v>
       </c>
       <c r="L46">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C47" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D47" t="s">
         <v>2</v>
@@ -2460,11 +2418,11 @@
       <c r="I47">
         <v>0</v>
       </c>
-      <c r="J47">
-        <v>-199.13333333333333</v>
-      </c>
-      <c r="K47">
-        <v>7.9122268251948746</v>
+      <c r="J47" s="2">
+        <v>-256.83333333333331</v>
+      </c>
+      <c r="K47" s="2">
+        <v>9.6738479072876338</v>
       </c>
       <c r="L47">
         <v>3</v>
@@ -2472,313 +2430,356 @@
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
+        <v>19</v>
+      </c>
+      <c r="C48" t="s">
+        <v>20</v>
+      </c>
+      <c r="D48">
+        <v>653.01</v>
+      </c>
+      <c r="E48">
+        <v>56.766532393656014</v>
+      </c>
+      <c r="F48">
+        <v>2</v>
+      </c>
+      <c r="G48">
+        <v>20.49</v>
+      </c>
+      <c r="H48" t="s">
+        <v>2</v>
+      </c>
+      <c r="I48">
+        <v>1</v>
+      </c>
+      <c r="J48" s="2">
+        <v>-274.8</v>
+      </c>
+      <c r="K48" s="2">
+        <v>2.4331050121192805</v>
+      </c>
+      <c r="L48">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>58</v>
+      </c>
+      <c r="C49" t="s">
+        <v>72</v>
+      </c>
+      <c r="D49" t="s">
+        <v>2</v>
+      </c>
+      <c r="E49" t="s">
+        <v>2</v>
+      </c>
+      <c r="F49">
+        <v>0</v>
+      </c>
+      <c r="G49" t="s">
+        <v>2</v>
+      </c>
+      <c r="H49" t="s">
+        <v>2</v>
+      </c>
+      <c r="I49">
+        <v>0</v>
+      </c>
+      <c r="J49" s="2">
+        <v>-199.13333333333333</v>
+      </c>
+      <c r="K49" s="2">
+        <v>7.9122268251948746</v>
+      </c>
+      <c r="L49">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>7</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C50" t="s">
         <v>8</v>
       </c>
-      <c r="D48">
+      <c r="D50">
         <v>683</v>
       </c>
-      <c r="E48" t="s">
-        <v>2</v>
-      </c>
-      <c r="F48">
-        <v>1</v>
-      </c>
-      <c r="G48">
+      <c r="E50" t="s">
+        <v>2</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50">
         <v>37.200000000000003</v>
       </c>
-      <c r="H48" t="s">
-        <v>2</v>
-      </c>
-      <c r="I48">
-        <v>1</v>
-      </c>
-      <c r="J48">
+      <c r="H50" t="s">
+        <v>2</v>
+      </c>
+      <c r="I50">
+        <v>1</v>
+      </c>
+      <c r="J50" s="2">
         <v>-330.4</v>
       </c>
-      <c r="K48">
+      <c r="K50" s="2">
         <v>1.4071247279470325</v>
       </c>
-      <c r="L48">
+      <c r="L50">
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>59</v>
+      </c>
+      <c r="C51" t="s">
+        <v>73</v>
+      </c>
+      <c r="D51">
+        <v>376.15</v>
+      </c>
+      <c r="E51" t="s">
+        <v>2</v>
+      </c>
+      <c r="F51">
+        <v>1</v>
+      </c>
+      <c r="G51">
+        <v>41.421600000000005</v>
+      </c>
+      <c r="H51" t="s">
+        <v>2</v>
+      </c>
+      <c r="I51">
+        <v>1</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>60</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C52" t="s">
         <v>74</v>
       </c>
-      <c r="D49">
-        <v>376.15</v>
-      </c>
-      <c r="E49" t="s">
-        <v>2</v>
-      </c>
-      <c r="F49">
-        <v>1</v>
-      </c>
-      <c r="G49">
-        <v>41.421600000000005</v>
-      </c>
-      <c r="H49" t="s">
-        <v>2</v>
-      </c>
-      <c r="I49">
-        <v>1</v>
-      </c>
-      <c r="J49" t="s">
-        <v>2</v>
-      </c>
-      <c r="K49" t="s">
-        <v>2</v>
-      </c>
-      <c r="L49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+      <c r="D52">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="E52" t="s">
+        <v>2</v>
+      </c>
+      <c r="F52">
+        <v>1</v>
+      </c>
+      <c r="G52">
+        <v>1.29704</v>
+      </c>
+      <c r="H52" t="s">
+        <v>2</v>
+      </c>
+      <c r="I52">
+        <v>1</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K52" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>61</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C53" t="s">
         <v>75</v>
       </c>
-      <c r="D50">
-        <v>295.14999999999998</v>
-      </c>
-      <c r="E50" t="s">
-        <v>2</v>
-      </c>
-      <c r="F50">
-        <v>1</v>
-      </c>
-      <c r="G50">
-        <v>1.29704</v>
-      </c>
-      <c r="H50" t="s">
-        <v>2</v>
-      </c>
-      <c r="I50">
-        <v>1</v>
-      </c>
-      <c r="J50" t="s">
-        <v>2</v>
-      </c>
-      <c r="K50" t="s">
-        <v>2</v>
-      </c>
-      <c r="L50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+      <c r="D53">
+        <v>412.15</v>
+      </c>
+      <c r="E53" t="s">
+        <v>2</v>
+      </c>
+      <c r="F53">
+        <v>1</v>
+      </c>
+      <c r="G53">
+        <v>39.329600000000006</v>
+      </c>
+      <c r="H53" t="s">
+        <v>2</v>
+      </c>
+      <c r="I53">
+        <v>1</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>62</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C54" t="s">
         <v>76</v>
       </c>
-      <c r="D51">
-        <v>412.15</v>
-      </c>
-      <c r="E51" t="s">
-        <v>2</v>
-      </c>
-      <c r="F51">
-        <v>1</v>
-      </c>
-      <c r="G51">
-        <v>39.329600000000006</v>
-      </c>
-      <c r="H51" t="s">
-        <v>2</v>
-      </c>
-      <c r="I51">
-        <v>1</v>
-      </c>
-      <c r="J51" t="s">
-        <v>2</v>
-      </c>
-      <c r="K51" t="s">
-        <v>2</v>
-      </c>
-      <c r="L51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+      <c r="D54" t="s">
+        <v>2</v>
+      </c>
+      <c r="E54" t="s">
+        <v>2</v>
+      </c>
+      <c r="F54">
+        <v>0</v>
+      </c>
+      <c r="G54" t="s">
+        <v>2</v>
+      </c>
+      <c r="H54" t="s">
+        <v>2</v>
+      </c>
+      <c r="I54">
+        <v>0</v>
+      </c>
+      <c r="J54" s="2">
+        <v>-442</v>
+      </c>
+      <c r="K54" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L54">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>21</v>
+      </c>
+      <c r="C55" t="s">
+        <v>22</v>
+      </c>
+      <c r="D55">
+        <v>459.61</v>
+      </c>
+      <c r="E55">
+        <v>61.461721420734726</v>
+      </c>
+      <c r="F55">
+        <v>2</v>
+      </c>
+      <c r="G55">
+        <v>66.58</v>
+      </c>
+      <c r="H55" t="s">
+        <v>2</v>
+      </c>
+      <c r="I55">
+        <v>1</v>
+      </c>
+      <c r="J55" s="2">
+        <v>-487.5</v>
+      </c>
+      <c r="K55" s="2">
+        <v>17.677669529663689</v>
+      </c>
+      <c r="L55">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>63</v>
       </c>
-      <c r="C52" t="s">
+      <c r="C56" t="s">
         <v>77</v>
       </c>
-      <c r="D52" t="s">
-        <v>2</v>
-      </c>
-      <c r="E52" t="s">
-        <v>2</v>
-      </c>
-      <c r="F52">
-        <v>0</v>
-      </c>
-      <c r="G52" t="s">
-        <v>2</v>
-      </c>
-      <c r="H52" t="s">
-        <v>2</v>
-      </c>
-      <c r="I52">
-        <v>0</v>
-      </c>
-      <c r="J52">
-        <v>-442</v>
-      </c>
-      <c r="K52" t="s">
-        <v>2</v>
-      </c>
-      <c r="L52">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>21</v>
-      </c>
-      <c r="C53" t="s">
-        <v>22</v>
-      </c>
-      <c r="D53">
-        <v>459.61</v>
-      </c>
-      <c r="E53">
-        <v>61.461721420734726</v>
-      </c>
-      <c r="F53">
-        <v>2</v>
-      </c>
-      <c r="G53">
-        <v>66.58</v>
-      </c>
-      <c r="H53" t="s">
-        <v>2</v>
-      </c>
-      <c r="I53">
-        <v>1</v>
-      </c>
-      <c r="J53">
-        <v>-487.5</v>
-      </c>
-      <c r="K53">
-        <v>17.677669529663689</v>
-      </c>
-      <c r="L53">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>64</v>
-      </c>
-      <c r="C54" t="s">
-        <v>78</v>
-      </c>
-      <c r="D54" t="s">
-        <v>2</v>
-      </c>
-      <c r="E54" t="s">
-        <v>2</v>
-      </c>
-      <c r="F54">
-        <v>0</v>
-      </c>
-      <c r="G54" t="s">
-        <v>2</v>
-      </c>
-      <c r="H54" t="s">
-        <v>2</v>
-      </c>
-      <c r="I54">
-        <v>0</v>
-      </c>
-      <c r="J54">
+      <c r="D56" t="s">
+        <v>2</v>
+      </c>
+      <c r="E56" t="s">
+        <v>2</v>
+      </c>
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="G56" t="s">
+        <v>2</v>
+      </c>
+      <c r="H56" t="s">
+        <v>2</v>
+      </c>
+      <c r="I56">
+        <v>0</v>
+      </c>
+      <c r="J56" s="2">
         <v>-395</v>
       </c>
-      <c r="K54" t="s">
-        <v>2</v>
-      </c>
-      <c r="L54">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="55" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+      <c r="K56" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="L56">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>41</v>
       </c>
-      <c r="C55" t="s">
+      <c r="C57" t="s">
         <v>42</v>
       </c>
-      <c r="D55">
+      <c r="D57">
         <v>153.26</v>
       </c>
-      <c r="E55">
+      <c r="E57">
         <v>3.6390932936653244</v>
       </c>
-      <c r="F55">
+      <c r="F57">
         <v>5</v>
       </c>
-      <c r="G55">
+      <c r="G57">
         <v>6.5419999999999998</v>
       </c>
-      <c r="H55">
+      <c r="H57">
         <v>2.8284271247458787E-3</v>
       </c>
-      <c r="I55">
-        <v>2</v>
-      </c>
-      <c r="J55">
+      <c r="I57">
+        <v>2</v>
+      </c>
+      <c r="J57" s="2">
         <v>-27.2</v>
       </c>
-      <c r="K55">
+      <c r="K57" s="2">
         <v>4.9497474683058327</v>
       </c>
-      <c r="L55">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A56" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C56" t="s">
-        <v>44</v>
-      </c>
-      <c r="D56">
-        <f>273.15+286</f>
-        <v>559.15</v>
-      </c>
-      <c r="G56">
-        <f>O56/1000</f>
-        <v>7.14</v>
-      </c>
-      <c r="J56">
-        <f>P56/1000</f>
-        <v>-190.8</v>
-      </c>
-      <c r="O56">
-        <f>AVERAGE(7.56,6.72)*1000</f>
-        <v>7140</v>
-      </c>
-      <c r="P56">
-        <v>-190800</v>
+      <c r="L57">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A2:A20">
+  <conditionalFormatting sqref="A2:A57">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>AND(F2&gt;0,I2&gt;0,L2&gt;0)</formula>
     </cfRule>
@@ -2787,6 +2788,5 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>